<commit_message>
vault backup: 2026-07-13 20:14:47
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -27,237 +27,237 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="16"/>
-      <color rgb="001F4E79"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-      <color rgb="00000000"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="00000000"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-      <color rgb="001F4E79"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-      <color rgb="00FFFFFF"/>
-      <name val="等线"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="10"/>
-      <color rgb="00000000"/>
-      <name val="等线"/>
-    </font>
-  </fonts>
-  <fills count="4">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="6">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00BFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00BFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00BFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00BFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="0"/>
+  <x:fonts count="7">
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b val="1"/>
+      <x:sz val="16"/>
+      <x:color rgb="001F4E79"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:b val="1"/>
+      <x:sz val="11"/>
+      <x:color rgb="00000000"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="00000000"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:b val="1"/>
+      <x:sz val="12"/>
+      <x:color rgb="001F4E79"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:b val="1"/>
+      <x:sz val="11"/>
+      <x:color rgb="00FFFFFF"/>
+      <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:b val="1"/>
+      <x:sz val="10"/>
+      <x:color rgb="00000000"/>
+      <x:name val="等线"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="4">
+    <x:fill>
+      <x:patternFill/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="00DDEBF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="00305496"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="6">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00BFBFBF"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="10">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </x:cellStyles>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <x:colors>
+    <x:indexedColors>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008000"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00808000"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="00C0C0C0"/>
+      <x:rgbColor rgb="00808080"/>
+      <x:rgbColor rgb="009999FF"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00FFFFCC"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00660066"/>
+      <x:rgbColor rgb="00FF8080"/>
+      <x:rgbColor rgb="000066CC"/>
+      <x:rgbColor rgb="00CCCCFF"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="0000CCFF"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00CCFFCC"/>
+      <x:rgbColor rgb="00FFFF99"/>
+      <x:rgbColor rgb="0099CCFF"/>
+      <x:rgbColor rgb="00FF99CC"/>
+      <x:rgbColor rgb="00CC99FF"/>
+      <x:rgbColor rgb="00FFCC99"/>
+      <x:rgbColor rgb="003366FF"/>
+      <x:rgbColor rgb="0033CCCC"/>
+      <x:rgbColor rgb="0099CC00"/>
+      <x:rgbColor rgb="00FFCC00"/>
+      <x:rgbColor rgb="00FF9900"/>
+      <x:rgbColor rgb="00FF6600"/>
+      <x:rgbColor rgb="00666699"/>
+      <x:rgbColor rgb="00969696"/>
+      <x:rgbColor rgb="00003366"/>
+      <x:rgbColor rgb="00339966"/>
+      <x:rgbColor rgb="00003300"/>
+      <x:rgbColor rgb="00333300"/>
+      <x:rgbColor rgb="00993300"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00333399"/>
+      <x:rgbColor rgb="00333333"/>
+    </x:indexedColors>
+  </x:colors>
+</x:styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -601,10 +601,8 @@
           <x:t>追溯依据</x:t>
         </x:is>
       </x:c>
-      <x:c r="B5" s="3" t="inlineStr">
-        <x:is>
-          <x:t>软件需求规格说明.md（SRS V3.3）</x:t>
-        </x:is>
+      <x:c r="B5" s="3" t="str">
+        <x:v>软件需求规格说明.md（SRS V3.4）</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n"/>
       <x:c r="D5" s="4" t="n"/>
@@ -1227,10 +1225,8 @@
           <x:t>对采集任务进行有序调度，保证采得不重复、不丢失、不失控——基于 Redis 实现任务与 URL 去重、调度队列与分布式锁，并对采集范围、频率、并发设配额上限超限自动限流，支撑情报回注入池去重与配额约束（II-15）。</x:t>
         </x:is>
       </x:c>
-      <x:c r="F4" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 爬虫 K3s/Kafka/Redis（任务去重与限流）</x:t>
-        </x:is>
+      <x:c r="F4" s="3" t="str">
+        <x:v>需求.md 爬虫 K8s(KubeSphere)/Kafka/Redis（任务去重与限流）</x:v>
       </x:c>
       <x:c r="G4" s="3" t="inlineStr">
         <x:is>
@@ -1402,10 +1398,8 @@
           <x:t>DC 数据爬取子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E7" s="3" t="inlineStr">
-        <x:is>
-          <x:t>将清洗后的结构化数据按数据特征持久化到不同的存储模型——明细数据入 HBase 列式库、元数据与索引入关系库、关系数据入图库，供后续分析与检索按需读取。</x:t>
-        </x:is>
+      <x:c r="E7" s="3" t="str">
+        <x:v>将清洗后的结构化数据按数据特征持久化到不同的存储模型——明细数据入 ClickHouse 列式库、元数据与索引入关系库、关系数据入 NebulaGraph 图库，供后续分析与检索按需读取。</x:v>
       </x:c>
       <x:c r="F7" s="3" t="inlineStr">
         <x:is>
@@ -1432,10 +1426,8 @@
           <x:t>功能测试</x:t>
         </x:is>
       </x:c>
-      <x:c r="K7" s="3" t="inlineStr">
-        <x:is>
-          <x:t>清洗后结果可正确写入 HBase、关系库与图数据库；写入失败可进入重试队列重试。</x:t>
-        </x:is>
+      <x:c r="K7" s="3" t="str">
+        <x:v>清洗后结果可正确写入 ClickHouse、关系库与 NebulaGraph 图库；写入失败可进入重试队列重试。</x:v>
       </x:c>
       <x:c r="L7" s="6" t="inlineStr">
         <x:is>
@@ -6264,10 +6256,8 @@
           <x:t>业务数据</x:t>
         </x:is>
       </x:c>
-      <x:c r="D9" s="3" t="inlineStr">
-        <x:is>
-          <x:t>采集与 ETL 加工数据：ETL 结果存于 HBase，关系数据存于图数据库（限 DC 采集与清洗存储）</x:t>
-        </x:is>
+      <x:c r="D9" s="3" t="str">
+        <x:v>采集与 ETL 加工数据：ETL 明细结果存于 ClickHouse，关系数据存于 NebulaGraph 图库（限 DC 采集与清洗存储）</x:v>
       </x:c>
       <x:c r="E9" s="3" t="inlineStr">
         <x:is>
@@ -6607,15 +6597,11 @@
           <x:t>技术选型</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="3" t="inlineStr">
-        <x:is>
-          <x:t>爬虫与 ETL 应复用现有大数据与基础设施组件，包括 K3s（爬虫集群容器编排）、Kafka、Redis、Spark 与 HBase</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="3" t="inlineStr">
-        <x:is>
-          <x:t>R-DC-001~006（复用 K3s/Kafka/Redis/Spark/HBase）</x:t>
-        </x:is>
+      <x:c r="D4" s="3" t="str">
+        <x:v>爬虫与 ETL 应复用现有大数据与基础设施组件，包括 Kubernetes（由 KubeSphere 管理，爬虫集群容器编排）、Kafka、Redis、PySpark 与 ClickHouse</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="str">
+        <x:v>R-DC-001~006（复用 K8s/Kafka/Redis/PySpark/ClickHouse）</x:v>
       </x:c>
       <x:c r="F4" s="3" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
vault backup: 2026-07-13 21:15:27
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -602,21 +602,19 @@
         </x:is>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>软件需求规格说明.md（SRS V3.4）</x:v>
+        <x:v>软件需求规格说明.md（SRS V3.5）</x:v>
       </x:c>
       <x:c r="C5" s="4" t="n"/>
       <x:c r="D5" s="4" t="n"/>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="2" t="inlineStr">
         <x:is>
           <x:t>设计对应</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="3" t="inlineStr">
-        <x:is>
-          <x:t>软件概要设计-模块功能拆分-v2.xlsx（40 模块 / 146 功能）</x:t>
-        </x:is>
+      <x:c r="B6" s="3" t="str">
+        <x:v>软件概要设计说明.md V2.4 / 软件概要设计-模块功能拆分-v2.xlsx（40 模块 / 146 功能）/ 软件详细设计说明-DC子系统.md V1.2 / 软件详细设计说明-OM子系统.md V1.0</x:v>
       </x:c>
       <x:c r="C6" s="4" t="n"/>
       <x:c r="D6" s="4" t="n"/>
@@ -2439,10 +2437,8 @@
           <x:t>II-04 日志与指标上报接口。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J24" s="3" t="inlineStr">
-        <x:is>
-          <x:t>功能测试 + 演示</x:t>
-        </x:is>
+      <x:c r="J24" s="3" t="str">
+        <x:v>功能测试 + 演示（复用 KubeSphere 可观测底座，OM 只读查询代理 + 分析入仓；详见 OM SDD §5.1/§5.2/§6）</x:v>
       </x:c>
       <x:c r="K24" s="3" t="inlineStr">
         <x:is>
@@ -2484,10 +2480,8 @@
           <x:t>需求.md 运维监控（告警与运维）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-OM-03 告警引擎（告警大脑）；M-OM-04 运维可视化与作业（运维作业台）</x:t>
-        </x:is>
+      <x:c r="G25" s="3" t="str">
+        <x:v>M-OM-03 告警引擎（告警观测，只读观测 Alertmanager 规则/事件 + 事件归档）；M-OM-04 运维可视化与作业（运维作业台）</x:v>
       </x:c>
       <x:c r="H25" s="3" t="inlineStr">
         <x:is>
@@ -2499,10 +2493,8 @@
           <x:t>无（依赖 R-OM-001 时序指标数据）。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J25" s="3" t="inlineStr">
-        <x:is>
-          <x:t>功能测试 + 演示</x:t>
-        </x:is>
+      <x:c r="J25" s="3" t="str">
+        <x:v>功能测试 + 演示（告警规则配置由 KubeSphere 控制台承担，OM 只读观测；详见 OM SDD §5.3/§6）</x:v>
       </x:c>
       <x:c r="K25" s="3" t="inlineStr">
         <x:is>
@@ -4167,10 +4159,8 @@
           <x:t>R-MC-007 任务幂等重试、R-MC-005 熔断、R-DC-001 断点续采、R-MC-001 Agent 重连（M-MC-05/07、M-DC-02）</x:t>
         </x:is>
       </x:c>
-      <x:c r="F21" s="3" t="inlineStr">
-        <x:is>
-          <x:t>测试 + 分析</x:t>
-        </x:is>
+      <x:c r="F21" s="3" t="str">
+        <x:v>V2 演进验证（当前版本单副本，可用性目标在 V2 多副本 HA 演进后强制达标）</x:v>
       </x:c>
       <x:c r="G21" s="6" t="inlineStr">
         <x:is>
@@ -4272,10 +4262,8 @@
           <x:t>R-MC-007 任务幂等重试、R-MC-005 熔断、R-DC-001 断点续采、R-MC-001 Agent 重连（M-MC-05/07、M-DC-02）</x:t>
         </x:is>
       </x:c>
-      <x:c r="F24" s="3" t="inlineStr">
-        <x:is>
-          <x:t>测试 + 分析</x:t>
-        </x:is>
+      <x:c r="F24" s="3" t="str">
+        <x:v>V2 演进验证（当前版本单副本存在单点；V2 演进多副本 HA 后达标）</x:v>
       </x:c>
       <x:c r="G24" s="6" t="inlineStr">
         <x:is>

</xml_diff>

<commit_message>
vault backup: 2026-07-14 11:26:24
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:numFmts count="0"/>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -71,6 +71,13 @@
       <x:sz val="10"/>
       <x:color rgb="00000000"/>
       <x:name val="等线"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="00000000"/>
+      <x:name val="等线"/>
+      <x:family xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="2"/>
+      <x:scheme xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" val="minor"/>
     </x:font>
   </x:fonts>
   <x:fills count="4">
@@ -161,7 +168,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
@@ -182,6 +189,12 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -2541,25 +2554,19 @@
           <x:t>M-COM-01 身份认证（身份守门人）；M-COM-02 权限与组织管理（权限决策与组织隔离）</x:t>
         </x:is>
       </x:c>
-      <x:c r="H26" s="3" t="inlineStr">
-        <x:is>
-          <x:t>F-COM-01-01；F-COM-01-02；F-COM-01-03；F-COM-02-01；F-COM-02-02；F-COM-02-03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I26" s="3" t="inlineStr">
-        <x:is>
-          <x:t>无（各子系统统一调用）。</x:t>
-        </x:is>
+      <x:c r="H26" s="3" t="str">
+        <x:v>F-COM-01-01；F-COM-01-03；F-COM-02-01；F-COM-02-02；F-COM-02-03</x:v>
+      </x:c>
+      <x:c r="I26" s="3" t="str">
+        <x:v>II-16 COM 认证服务（M-COM-01）；II-17 COM 权限与组织管理（M-COM-02）；各子系统统一调用。</x:v>
       </x:c>
       <x:c r="J26" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试（认证授权、多组织隔离）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K26" s="3" t="inlineStr">
-        <x:is>
-          <x:t>登录认证与双因素可用；RBAC 权限决策可按角色控制；多组织数据可隔离且禁止跨组织访问。</x:t>
-        </x:is>
+      <x:c r="K26" s="3" t="str">
+        <x:v>登录认证可用；RBAC 权限决策可按角色控制；多组织数据可隔离且禁止跨组织访问。</x:v>
       </x:c>
       <x:c r="L26" s="6" t="inlineStr">
         <x:is>
@@ -4320,10 +4327,8 @@
           <x:t>安全性</x:t>
         </x:is>
       </x:c>
-      <x:c r="D26" s="3" t="inlineStr">
-        <x:is>
-          <x:t>系统应提供用户认证与双因素，并对全部 API 进行鉴权</x:t>
-        </x:is>
+      <x:c r="D26" s="3" t="str">
+        <x:v>系统应提供用户认证，并对全部 API 进行鉴权</x:v>
       </x:c>
       <x:c r="E26" s="3" t="inlineStr">
         <x:is>
@@ -5922,6 +5927,64 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="10">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" s="10" t="str">
+        <x:v>内部接口 II</x:v>
+      </x:c>
+      <x:c r="C25" s="10" t="str">
+        <x:v>II-16</x:v>
+      </x:c>
+      <x:c r="D25" s="11" t="str">
+        <x:v>COM 认证服务接口</x:v>
+      </x:c>
+      <x:c r="E25" s="11" t="str">
+        <x:v>公共功能 COM（M-COM-01）</x:v>
+      </x:c>
+      <x:c r="F25" s="11" t="str">
+        <x:v>各子系统 / 前端</x:v>
+      </x:c>
+      <x:c r="G25" s="11" t="str">
+        <x:v>入：账号密码；出：JWT 令牌（含 user_id/org_id/roles）。含登录、登出、令牌刷新。</x:v>
+      </x:c>
+      <x:c r="H25" s="11" t="str">
+        <x:v>R-COM-001</x:v>
+      </x:c>
+      <x:c r="I25" s="11" t="str">
+        <x:v>接口测试（认证）</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="10">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" s="10" t="str">
+        <x:v>内部接口 II</x:v>
+      </x:c>
+      <x:c r="C26" s="10" t="str">
+        <x:v>II-17</x:v>
+      </x:c>
+      <x:c r="D26" s="11" t="str">
+        <x:v>COM 权限与组织管理接口</x:v>
+      </x:c>
+      <x:c r="E26" s="11" t="str">
+        <x:v>公共功能 COM（M-COM-02）</x:v>
+      </x:c>
+      <x:c r="F26" s="11" t="str">
+        <x:v>各子系统 / 前端</x:v>
+      </x:c>
+      <x:c r="G26" s="11" t="str">
+        <x:v>入：用户/角色/组织配置；出：权限决策结果、组织结构。含用户/角色/组织 CRUD、账号解锁、RBAC 权限点查询。</x:v>
+      </x:c>
+      <x:c r="H26" s="11" t="str">
+        <x:v>R-COM-001</x:v>
+      </x:c>
+      <x:c r="I26" s="11" t="str">
+        <x:v>接口测试（权限组织）</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:autoFilter ref="A1:J24"/>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-14 17:45:39
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -5944,6 +5944,38 @@
       </x:c>
     </x:row>
     <x:row r="26">
+      <x:c r="A26">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>内部接口 II</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>II-18</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>用户画像查询接口</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>舆情作战 OCC</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>蜂群 SWM</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>入：用户画像查询请求（account_id 或目标标识）；出：用户画像（来源于 OCC R-OCC-004 全维度档案，含身份特征、立场倾向、兴趣领域等）</x:v>
+      </x:c>
+      <x:c r="H26" t="str">
+        <x:v>R-SWM-005；R-OCC-004</x:v>
+      </x:c>
+      <x:c r="I26" t="str">
+        <x:v>接口测试</x:v>
+      </x:c>
+      <x:c r="J26" t="str">
+        <x:v>✓ 完整</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
       <x:c r="A26" s="10">
         <x:v>24</x:v>
       </x:c>
@@ -6397,20 +6429,14 @@
           <x:t>业务数据-智能体</x:t>
         </x:is>
       </x:c>
-      <x:c r="D12" s="3" t="inlineStr">
-        <x:is>
-          <x:t>蜂群智能体数据：以 agent_id 为标识的智能体定义（人设标签、提示词、记忆、作业策略）及与 account_id 的 1:1 绑定关系、作业记忆与提示词模板版本</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="3" t="inlineStr">
-        <x:is>
-          <x:t>蜂群 SWM（定义）/群控 MC（持存）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F12" s="3" t="inlineStr">
-        <x:is>
-          <x:t>R-SWM-001/002/003；R-MC-013/014（智能体数据）</x:t>
-        </x:is>
+      <x:c r="D12" s="3" t="str">
+        <x:v>蜂群智能体数据：以 agent_id（稳定逻辑标识）为索引的提示词包（人设标签、提示词、作业策略及当前生效版本号）及与 account_id 的 1:1 绑定关系、智能体作业记忆（Java 记忆服务 swm-memory 承载）与提示词模板版本</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>蜂群 SWM（提示词包生成/记忆承载）/群控 MC（提示词包持存）</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:v>R-SWM-001/002/003/005；R-MC-013/014（智能体数据）</x:v>
       </x:c>
       <x:c r="G12" s="6" t="inlineStr">
         <x:is>
@@ -6876,10 +6902,8 @@
           <x:t>架构约束</x:t>
         </x:is>
       </x:c>
-      <x:c r="D11" s="3" t="inlineStr">
-        <x:is>
-          <x:t>智能体模式下的视觉推理应调用 IRS 本地大模型，不经执行网关；推理产出的动作指令再经执行网关落地</x:t>
-        </x:is>
+      <x:c r="D11" s="3" t="str">
+        <x:v>智能体模式下由群控子系统（MC）的 agent-runtime 子模块调用 IRS 本地大模型完成视觉推理，不经 MC 执行网关；推理产出的动作指令再经执行网关落地。agent-runtime 与执行网关逻辑隔离，以保持推理与执行分离语义</x:v>
       </x:c>
       <x:c r="E11" s="3" t="inlineStr">
         <x:is>
@@ -6911,15 +6935,11 @@
           <x:t>架构约束</x:t>
         </x:is>
       </x:c>
-      <x:c r="D12" s="3" t="inlineStr">
-        <x:is>
-          <x:t>执行层职责应按"统一执行网关 + 内容权威源"两类归属：指纹浏览器 Profile 的管理（创建、指纹固化、接入、监控）与桌面端 CDP 执行网关、移动端终端管理与 ADB/无障碍执行网关、账号主数据（注册、凭据、验证、风险评估、生命周期、账号分类）的唯一维护与共享分发、智能体执行宿主，均归群控子系统（MC）；内容资源（素材入库、分类、审核、排期、分发）唯一权威源归舆情作战业务子系统（OCC）。蜂群智能体子系统（SWM）作为智能体定义与记忆中心，将智能体定义同步至 MC 持存；舆情作战子系统（OCC）以作战编排方式直接编排 MC 中的智能体节点与自动化脚本节点，使执行终端管理、账号主数据与动作执行统一收口</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="3" t="inlineStr">
-        <x:is>
-          <x:t>R-MC-001/005/011/014；R-OCC-009（执行层职责归属）</x:t>
-        </x:is>
+      <x:c r="D12" s="3" t="str">
+        <x:v>执行层职责应按 统一执行网关 + 内容权威源 两类归属：指纹浏览器 Profile 的管理（创建、指纹固化、接入、监控）与桌面端 CDP 执行网关、移动端终端管理与 ADB/无障碍执行网关、账号主数据（注册、凭据、验证、风险评估、生命周期、账号分类）的唯一维护与共享分发、智能体执行宿主（含运行时 agent-runtime 子模块），均归群控子系统（MC）；内容资源（素材入库、分类、审核、排期、分发）唯一权威源归舆情作战业务子系统（OCC）。蜂群智能体子系统（SWM）作为提示词生成与记忆中心，将生成的提示词包（人设标签、提示词、作业策略）同步至 MC 持存，运行时（场景适配、动态调用、调用 IRS 推理）归 MC 的 agent-runtime 子模块；舆情作战子系统（OCC）以作战编排方式直接编排 MC 中的智能体节点与自动化脚本节点，使执行终端管理、账号主数据与动作执行统一收口</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>R-MC-001/005/006/011/014；R-OCC-009（执行层职责归属）</x:v>
       </x:c>
       <x:c r="F12" s="3" t="inlineStr">
         <x:is>
@@ -6997,6 +7017,64 @@
         </x:is>
       </x:c>
       <x:c r="G14" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>CON-14</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>技术选型</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>蜂群智能体子系统（SWM）的提示词工程（模板库、版本管理、Playground 试运行、版本输出对比）与智能体评测（评测集、评估器、实验）能力，以开源项目 coze-loop（Go）作为提示词工程与评测引擎旁挂集成；其余智能体域组件（网关、编排提炼、记忆服务）采用 Java（Spring Boot），与管控/业务微服务统一 Java 栈一致。coze-loop 作为唯一外部 Go 服务，经 HTTP/OpenAPI 与 Java 侧解耦（智能体域特例，仿 DC 采集域特例思路）</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>R-SWM-001/002/004/005（智能体域技术选型特例）</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>评审 / 接口测试</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>✓ 完整</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="6" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>CON-13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="6" t="inlineStr">
+        <x:is>
+          <x:t>架构约束</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="3" t="inlineStr">
+        <x:is>
+          <x:t>账号应按用途分类管理：爬虫账号以桌面端指纹浏览器 Profile 为执行终端、其养护（养号）动作执行经 MC 统一执行网关的 CDP 通道，认知作战账号以移动端设备为执行终端、经 MC 统一执行网关的 ADB/无障碍通道执行养号动作；两类账号的注册、验证与生命周期等主数据均由群控子系统（MC）统一维护并向各子系统分发 account_id。账号-终端-代理绑定遵循差异化规则：真机、云手机、虚拟化真机执行"一设备一账号一 IP"，指纹浏览器 Profile 执行"一 Profile 一账号一 IP"（实例可多开），每个终端/Profile 绑定一个固定代理 IP</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="3" t="inlineStr">
+        <x:is>
+          <x:t>R-MC-009/011（账号分类与一设备一账号一 IP/一 Profile 一账号一 IP）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="3" t="inlineStr">
+        <x:is>
+          <x:t>功能测试</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="6" t="inlineStr">
         <x:is>
           <x:t>✓ 完整</x:t>
         </x:is>
@@ -7199,17 +7277,17 @@
           <x:t>蜂群智能体子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="C8" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="F8" s="6" t="n">
-        <x:v>4</x:v>
+      <x:c r="C8" s="6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D8" s="6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E8" s="6">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F8" s="6">
+        <x:v>5</x:v>
       </x:c>
       <x:c r="G8" s="6" t="inlineStr">
         <x:is>
@@ -7281,22 +7359,20 @@
           <x:t>合计</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="9" t="inlineStr">
-        <x:is>
-          <x:t>39 项功能需求</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C11" s="8" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="D11" s="8" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="E11" s="8" t="n">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F11" s="8" t="n">
-        <x:v>39</x:v>
+      <x:c r="B11" s="9" t="str">
+        <x:v>40 项功能需求</x:v>
+      </x:c>
+      <x:c r="C11" s="8">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D11" s="8">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E11" s="8">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="F11" s="8">
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G11" s="8" t="inlineStr">
         <x:is>
@@ -7349,10 +7425,8 @@
           <x:t>R-XX-NNN</x:t>
         </x:is>
       </x:c>
-      <x:c r="C16" s="6" t="inlineStr">
-        <x:is>
-          <x:t>39</x:t>
-        </x:is>
+      <x:c r="C16" s="6">
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D16" s="3" t="inlineStr">
         <x:is>
@@ -7484,10 +7558,8 @@
           <x:t>CON-NN</x:t>
         </x:is>
       </x:c>
-      <x:c r="C21" s="6" t="inlineStr">
-        <x:is>
-          <x:t>13</x:t>
-        </x:is>
+      <x:c r="C21" s="6">
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D21" s="3" t="inlineStr">
         <x:is>
@@ -7508,10 +7580,8 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
-      <x:c r="A24" s="3" t="inlineStr">
-        <x:is>
-          <x:t>1. 39 项功能需求（R-DC-001~008、R-MC-001~014、R-OM-001~002、R-COM-001、R-SWM-001~004、R-IRS-001、R-OCC-001~009）均已建立「上游来源→需求→概要设计模块/功能点→验证方法」完整追溯链。</x:t>
-        </x:is>
+      <x:c r="A24" s="3" t="str">
+        <x:v>1. 40 项功能需求（R-DC-001~008、R-MC-001~014、R-OM-001~002、R-COM-001、R-SWM-001~005、R-IRS-001、R-OCC-001~009）均已建立「上游来源→需求→概要设计模块/功能点→验证方法」完整追溯链。</x:v>
       </x:c>
       <x:c r="B24" s="4" t="n"/>
       <x:c r="C24" s="4" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-17 13:49:35
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -586,10 +586,8 @@
           <x:t>项目名称</x:t>
         </x:is>
       </x:c>
-      <x:c r="B3" s="3" t="inlineStr">
-        <x:is>
-          <x:t>认知作战平台（v1.0）</x:t>
-        </x:is>
+      <x:c r="B3" s="3" t="str">
+        <x:v>认知行动平台（v1.0）</x:v>
       </x:c>
       <x:c r="C3" s="4" t="n"/>
       <x:c r="D3" s="4" t="n"/>
@@ -2065,10 +2063,8 @@
           <x:t>MC 多设备矩阵自动化群控子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E18" s="3" t="inlineStr">
-        <x:is>
-          <x:t>承载养号、账号-终端-代理绑定、登录状态维护等可自动化的账号操作的执行编排，以及养号拟人化节奏策略（内置）。认知作战账号经移动端 ADB/无障碍通道养号、爬虫账号经桌面端 CDP 通道养护。养号等风控敏感场景可优先采用脚本模式编排。</x:t>
-        </x:is>
+      <x:c r="E18" s="3" t="str">
+        <x:v>承载养号、账号-终端-代理绑定、登录状态维护等可自动化的账号操作的执行编排，以及养号拟人化节奏策略（内置）。认知行动账号经移动端 ADB/无障碍通道养号、爬虫账号经桌面端 CDP 通道养护。养号等风控敏感场景可优先采用脚本模式编排。</x:v>
       </x:c>
       <x:c r="F18" s="3" t="inlineStr">
         <x:is>
@@ -2145,10 +2141,8 @@
           <x:t>F-MC-10-01；F-MC-10-02；F-MC-10-03；F-MC-10-04；F-MC-10-05；F-MC-10-06；F-MC-10-07；F-MC-10-08；F-MC-10-09</x:t>
         </x:is>
       </x:c>
-      <x:c r="I19" s="3" t="inlineStr">
-        <x:is>
-          <x:t>II-04 日志指标上报（至 OM）、II-10 作战编排下发与执行回传（效果回传 OCC）。</x:t>
-        </x:is>
+      <x:c r="I19" s="3" t="str">
+        <x:v>II-04 日志指标上报（至 OM）、II-10 行动编排下发与执行回传（效果回传 OCC）。</x:v>
       </x:c>
       <x:c r="J19" s="3" t="inlineStr">
         <x:is>
@@ -2305,20 +2299,16 @@
           <x:t>MC 多设备矩阵自动化群控子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E22" s="3" t="inlineStr">
-        <x:is>
-          <x:t>维护账号与智能体定义（agent_id）的严格 1:1 绑定关系，叠加账号-终端-代理绑定规则形成四元作战单元（agent_id:account_id:终端:代理 IP = 1:1:1:1）；并在账号被封禁后支持运营人员发起资产迁移，将原 agent_id 的人设标签、提示词版本与记忆整体继承到新账号，保证人格连贯性。</x:t>
-        </x:is>
+      <x:c r="E22" s="3" t="str">
+        <x:v>维护账号与智能体定义（agent_id）的严格 1:1 绑定关系，叠加账号-终端-代理绑定规则形成四元行动单元（agent_id:account_id:终端:代理 IP = 1:1:1:1）；并在账号被封禁后支持运营人员发起资产迁移，将原 agent_id 的提示词版本与记忆整体继承到新账号，保证行为连贯性。</x:v>
       </x:c>
       <x:c r="F22" s="3" t="inlineStr">
         <x:is>
           <x:t>智能体-账号 1:1 绑定与封号资产迁移</x:t>
         </x:is>
       </x:c>
-      <x:c r="G22" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-MC-13 智能体账号绑定与资产迁移（四元作战单元）</x:t>
-        </x:is>
+      <x:c r="G22" s="3" t="str">
+        <x:v>M-MC-13 智能体账号绑定与资产迁移（四元行动单元）</x:v>
       </x:c>
       <x:c r="H22" s="3" t="inlineStr">
         <x:is>
@@ -2335,10 +2325,8 @@
           <x:t>功能测试（1:1 绑定、封号资产迁移）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K22" s="3" t="inlineStr">
-        <x:is>
-          <x:t>agent_id↔account_id 1:1 绑定关系可记录与查询；四元作战单元可形成；封号资产可经人工触发整体迁移到新账号并延续人格。</x:t>
-        </x:is>
+      <x:c r="K22" s="3" t="str">
+        <x:v>agent_id↔account_id 1:1 绑定关系可记录与查询；四元行动单元可形成；封号资产可经人工触发整体迁移到新账号并延续行为。</x:v>
       </x:c>
       <x:c r="L22" s="6" t="inlineStr">
         <x:is>
@@ -2365,10 +2353,8 @@
           <x:t>MC 多设备矩阵自动化群控子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E23" s="3" t="inlineStr">
-        <x:is>
-          <x:t>作为智能体的执行宿主，接收并持存蜂群智能体子系统（SWM）同步来的智能体定义（以 agent_id 为标识，含人设标签、提示词、记忆、作业策略），在任务执行时调用这些定义驱动设备作业，并在执行前校验人设一致性。本功能确立"SWM 为智能体定义与记忆中心、MC 为智能体执行宿主"的分工。</x:t>
-        </x:is>
+      <x:c r="E23" s="3" t="str">
+        <x:v>作为智能体的执行宿主，接收并持存蜂群智能体子系统（SWM）同步来的提示词包（以 agent_id 为标识，含提示词、作业策略），在任务执行时调用这些定义驱动设备作业，并在执行前校验行为风格一致性。本功能确立 SWM 生成提示词包、MC 持存并运行（agent-runtime）、OCC 编排引用 的分工。</x:v>
       </x:c>
       <x:c r="F23" s="3" t="inlineStr">
         <x:is>
@@ -2395,10 +2381,8 @@
           <x:t>功能测试（持存/四元绑定/人设一致性校验/调用/更新）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K23" s="3" t="inlineStr">
-        <x:is>
-          <x:t>可以 agent_id 接收并持存 SWM 同步的智能体定义；四元绑定关系（agent_id↔account_id↔终端↔代理 IP）可记录与查询；任务执行前可校验人设一致性且不一致时拒绝执行；任务执行时可按定义调用并经执行网关落地动作；智能体定义更新后可使用最新版本执行；可作为 OCC 作战编排的智能体节点来源（以 agent_id 引用）。</x:t>
-        </x:is>
+      <x:c r="K23" s="3" t="str">
+        <x:v>可以 agent_id 接收并持存 SWM 同步的智能体定义；四元绑定关系（agent_id↔account_id↔终端↔代理 IP）可记录与查询；任务执行前可校验行为风格一致性且不一致时拒绝执行；任务执行时可按定义调用并经执行网关落地动作；智能体定义更新后可使用最新版本执行；可作为 OCC 行动编排的智能体节点来源（以 agent_id 引用）。</x:v>
       </x:c>
       <x:c r="L23" s="6" t="inlineStr">
         <x:is>
@@ -2583,10 +2567,8 @@
           <x:t>R-SWM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" s="3" t="inlineStr">
-        <x:is>
-          <x:t>提示词与人设管理</x:t>
-        </x:is>
+      <x:c r="C27" s="3" t="str">
+        <x:v>提示词管理</x:v>
       </x:c>
       <x:c r="D27" s="6" t="inlineStr">
         <x:is>
@@ -2594,7 +2576,7 @@
         </x:is>
       </x:c>
       <x:c r="E27" s="3" t="str">
-        <x:v>管理驱动智能体作业的提示词与智能体人设标签，支持人设标签绑定、提示词模板库分类、版本管理、Playground 试运行调试、版本输出对比与迭代优化，并以 agent_id 为标识将完整的提示词包（人设标签、提示词、作业策略）同步至 MC 持存。人设标签挂在 agent_id 上（不直接挂 account_id），随提示词包同步；账号主数据由 MC 统一维护（R-MC-011）。运行时场景适配与动态调用归 MC 的 agent-runtime 子模块（见 R-MC-006/014）。</x:v>
+        <x:v>管理驱动智能体作业的提示词，支持提示词模板库分类、版本管理、Playground 试运行调试、版本输出对比与迭代优化，并以 agent_id 为标识将提示词包（提示词、作业策略）同步至 MC 持存。V3.9（ADR-001）废除人设标签实体，人设属性直接写进提示词文本。账号主数据由 MC 统一维护（R-MC-011）。运行时场景适配与动态调用归 MC 的 agent-runtime 子模块（见 R-MC-006/014）。</x:v>
       </x:c>
       <x:c r="F27" s="3" t="inlineStr">
         <x:is>
@@ -2602,7 +2584,7 @@
         </x:is>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>M-SWM-01 人设标签管理（智能体人格定义中心）；M-SWM-02 提示词模板库与版本管理（提示词资产管理）</x:v>
+        <x:v>M-SWM-01 提示词管理（V3.9 改：原人设标签管理废除，改提示词模板/版本管理）；M-SWM-02 提示词模板库与版本管理（提示词资产管理）</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
         <x:v>F-SWM-01-01；F-SWM-01-02；F-SWM-02-01；F-SWM-02-02；F-SWM-02-03；F-SWM-02-04</x:v>
@@ -2614,7 +2596,7 @@
         <x:v>功能测试（人设绑 agent_id、模板库、版本/Playground/对比）</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
-        <x:v>人设标签可绑定到 agent_id 且涵盖画像属性（不复制账号主数据）；提示词模板库可分类管理；版本可按 agent_id 对比回滚；可在 Playground 中填入提示词草稿即时调用 IRS 试运行并查看产出；可将不同版本提示词并排对比输出；可结合反馈与调优结果迭代优化；提示词包可以 agent_id 同步至 MC 持存。</x:v>
+        <x:v>提示词模板库可分类管理；版本可按 agent_id 对比回滚；可在 Playground 中填入提示词草稿即时调用 IRS 试运行并查看产出；可将不同版本提示词并排对比输出；可结合反馈与调优结果迭代优化；提示词包可以 agent_id 同步至 MC 持存。</x:v>
       </x:c>
       <x:c r="L27" s="6" t="inlineStr">
         <x:is>
@@ -2698,7 +2680,7 @@
         </x:is>
       </x:c>
       <x:c r="E29" s="3" t="str">
-        <x:v>根据人设标签（画像、账号属性）构建可作业的智能体——配置驱动作业的提示词与作业策略（目标、场景、边界），组装为提示词包（人设标签、提示词、作业策略）并以 agent_id（稳定逻辑标识）为标识，经内部接口 II-14 同步至群控子系统（MC）持存、供舆情作战子系统（OCC）作战编排引用。记忆不在提示词包内，由记忆服务独立承载。本功能确立 SWM 生成提示词包、MC 持存并运行（agent-runtime）、OCC 编排引用 的分工。</x:v>
+        <x:v>根据提示词（画像、账号属性）构建可作业的智能体——配置驱动作业的提示词与作业策略（目标、场景、边界），组装为提示词包（提示词、作业策略）并以 agent_id（稳定逻辑标识）为标识，经内部接口 II-14 同步至群控子系统（MC）持存、供舆情行动子系统（OCC）行动编排引用。记忆不在提示词包内，由记忆服务独立承载。本功能确立 SWM 生成提示词包、MC 持存并运行（agent-runtime）、OCC 编排引用 的分工。</x:v>
       </x:c>
       <x:c r="F29" s="3" t="inlineStr">
         <x:is>
@@ -2720,7 +2702,7 @@
         </x:is>
       </x:c>
       <x:c r="K29" s="3" t="str">
-        <x:v>可按人设标签构建提示词包并以 agent_id 为标识；提示词包须包含人设标签、提示词、作业策略三项必填要素，缺一不可构建；agent_id 为稳定逻辑标识、提示词版本可随重生成升级；可与 account_id 严格 1:1 绑定；提示词包可经 II-14 同步至 MC 持存并取得版本号且同步成功率不低于 99%；构建出的智能体可作为 OCC 作战编排的智能体节点来源。</x:v>
+        <x:v>可按提示词构建提示词包并以 agent_id 为标识；提示词包须包含提示词、作业策略三项必填要素，缺一不可构建；agent_id 为稳定逻辑标识、提示词版本可随重生成升级；可与 account_id 严格 1:1 绑定；提示词包可经 II-14 同步至 MC 持存并取得版本号且同步成功率不低于 99%；构建出的智能体可作为 OCC 行动编排的智能体节点来源。</x:v>
       </x:c>
       <x:c r="L29" s="6" t="inlineStr">
         <x:is>
@@ -2747,10 +2729,8 @@
           <x:t>SWM 蜂群智能体子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>对构建出的智能体（R-SWM-003）进行质量评测，采用「线上效果 + 离线数据集」双轨评测范式评估智能体的有效性、稳定性与合规性；离线评测以"评测集、评估器、实验"三类可管理实体组织——评测集承载测试用例，评估器承载可复用的打分逻辑，实验承载一次可追踪、可对比的评测运行，淘汰低效定义、迭代优化高价值定义，形成"构建→评测→迭代"的闭环，使智能体定义随作业实践持续演进。双轨评测互补印证：线上效果反映真实作战表现，离线数据集提供受控、可复现、可对比的质量基准，避免单一维度误判。</x:t>
-        </x:is>
+      <x:c r="E30" s="3" t="str">
+        <x:v>对构建出的智能体（R-SWM-003）进行质量评测，采用「线上效果 + 离线数据集」双轨评测范式评估智能体的有效性、稳定性与合规性；离线评测以"评测集、评估器、实验"三类可管理实体组织——评测集承载测试用例，评估器承载可复用的打分逻辑，实验承载一次可追踪、可对比的评测运行，淘汰低效定义、迭代优化高价值定义，形成"构建→评测→迭代"的闭环，使智能体定义随作业实践持续演进。双轨评测互补印证：线上效果反映真实行动表现，离线数据集提供受控、可复现、可对比的质量基准，避免单一维度误判。</x:v>
       </x:c>
       <x:c r="F30" s="3" t="inlineStr">
         <x:is>
@@ -2767,10 +2747,8 @@
           <x:t>F-SWM-06-01；F-SWM-06-02；F-SWM-06-03；F-SWM-06-04；F-SWM-06-05；F-SWM-06-06</x:t>
         </x:is>
       </x:c>
-      <x:c r="I30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>EI-05 本地大模型推理（离线跑题）、II-10 作战编排下发与执行回传（MC 作业效果数据来源）。</x:t>
-        </x:is>
+      <x:c r="I30" s="3" t="str">
+        <x:v>EI-05 本地大模型推理（离线跑题）、II-10 行动编排下发与执行回传（MC 作业效果数据来源）。</x:v>
       </x:c>
       <x:c r="J30" s="3" t="inlineStr">
         <x:is>
@@ -2796,31 +2774,31 @@
         <x:v>R-SWM-005</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
-        <x:v>提示词自动生成</x:v>
+        <x:v>对话编写提示词</x:v>
       </x:c>
       <x:c r="D31" s="6" t="str">
         <x:v>SWM 蜂群智能体子系统</x:v>
       </x:c>
       <x:c r="E31" s="3" t="str">
-        <x:v>根据账号属性与用户画像，经 IRS 本地大模型自动生成驱动智能体作业的提示词，降低人工编写成本并提升人设贴合度。用户画像来自 OCC 全维度档案（R-OCC-004），账号主数据来自 MC（II-01）；生成结果纳入版本管理并可作为 R-SWM-003 智能体构建的提示词来源。</x:v>
+        <x:v>用户上传画像素材或描述需求，经 IRS 本地大模型对话式辅助编写提示词（V3.9 改：ADR-001，不再经 II-01/II-18 系统拉取）；生成结果纳入版本管理并可作为 R-SWM-003 智能体构建的提示词来源。</x:v>
       </x:c>
       <x:c r="F31" s="3" t="str">
         <x:v>需求.md 蜂群智能体（提示词自动生成）</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>M-SWM-07 按账号与画像自动生成提示词（提示词自动生成引擎）</x:v>
+        <x:v>M-SWM-07 对话编写提示词（对话编写引擎）</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
         <x:v>F-SWM-07-01；F-SWM-07-02；F-SWM-07-03</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>II-01 账号服务接口（账号主数据）、II-18 用户画像查询接口（OCC 全维度档案）、EI-05 本地大模型推理（生成推理）。</x:v>
+        <x:v>EI-05 本地大模型推理（对话编写推理）。V3.9 删 II-01/II-18（不再系统拉取）。</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
-        <x:v>功能测试（账号+画像拉取、IRS 生成、版本化纳入构建）</x:v>
+        <x:v>功能测试（素材上传、对话编写、IRS 推理、版本化纳入构建）</x:v>
       </x:c>
       <x:c r="K31" s="3" t="str">
-        <x:v>可按 account_id 从 MC 拉取账号主数据；可按目标标识从 OCC 拉取用户画像（R-OCC-004 全维度档案）；可将账号属性与画像作为上下文经 IRS 生成提示词；生成结果可版本化并回写提示词库；生成结果可经人工审核微调后纳入 R-SWM-003 智能体构建。</x:v>
+        <x:v>可上传画像素材并描述需求；可与 IRS 对话式编写提示词；生成结果可版本化并回写提示词库；可经人工审核微调后纳入 R-SWM-003 智能体构建。</x:v>
       </x:c>
       <x:c r="L31" s="6" t="str">
         <x:v>✓ 完整</x:v>
@@ -2900,20 +2878,14 @@
           <x:t>目标识别与维护</x:t>
         </x:is>
       </x:c>
-      <x:c r="D33" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E33" s="3" t="inlineStr">
-        <x:is>
-          <x:t>识别舆情事件的目标要素并对其进行全生命周期维护。目标在系统中即数据对象——支持建档、修改、关联、状态流转与删除，而非一次识别即定型的只读结果。本能力融合情报侦察、多维画像与抓手挖掘中"识别目标"的部分：从舆情事件与传播数据中识别事件主体、传播源头、核心争议点、干预目标对象，并补充传播线索、事件/群体/账号/传播画像、干预切入点与薄弱点等目标属性，形成可持续维护的目标档案，为后续作战提供靶向。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F33" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 舆情作战（目标识别与维护）</x:t>
-        </x:is>
+      <x:c r="D33" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
+      </x:c>
+      <x:c r="E33" s="3" t="str">
+        <x:v>识别舆情事件的目标要素并对其进行全生命周期维护。目标在系统中即数据对象——支持建档、修改、关联、状态流转与删除，而非一次识别即定型的只读结果。本能力融合情报侦察、多维画像与抓手挖掘中\"识别目标\"的部分：从舆情事件与传播数据中识别事件主体、传播源头、核心争议点、干预目标对象，并补充传播线索、事件/群体/账号/传播画像、干预切入点与薄弱点等目标属性，形成可持续维护的目标档案，为后续行动提供靶向。</x:v>
+      </x:c>
+      <x:c r="F33" s="3" t="str">
+        <x:v>需求.md 舆情行动（目标识别与维护）</x:v>
       </x:c>
       <x:c r="G33" s="3" t="inlineStr">
         <x:is>
@@ -2960,10 +2932,8 @@
           <x:t>群体-个体下钻筛选</x:t>
         </x:is>
       </x:c>
-      <x:c r="D34" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="D34" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E34" s="3" t="inlineStr">
         <x:is>
@@ -3020,10 +2990,8 @@
           <x:t>关系图谱与图查询</x:t>
         </x:is>
       </x:c>
-      <x:c r="D35" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="D35" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E35" s="3" t="inlineStr">
         <x:is>
@@ -3080,10 +3048,8 @@
           <x:t>实体检索与档案</x:t>
         </x:is>
       </x:c>
-      <x:c r="D36" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="D36" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E36" s="3" t="inlineStr">
         <x:is>
@@ -3140,10 +3106,8 @@
           <x:t>文本智能分析</x:t>
         </x:is>
       </x:c>
-      <x:c r="D37" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="D37" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E37" s="3" t="inlineStr">
         <x:is>
@@ -3195,40 +3159,28 @@
           <x:t>R-OCC-006</x:t>
         </x:is>
       </x:c>
-      <x:c r="C38" s="3" t="inlineStr">
-        <x:is>
-          <x:t>作战编排</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D38" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E38" s="3" t="inlineStr">
-        <x:is>
-          <x:t>根据目标档案与干预切入点匹配干预策略、生成作业方案，并以"作战编排"的方式直接编排群控子系统（MC）中的执行节点形成执行流程（图）落地，形成"目标→编排→执行"的闭环。OCC 直接编排 MC 中的节点，蜂群智能体子系统（SWM）作为"智能体节点的供给方之一"参与编排。编排的节点类型本期为两类——智能体节点（其智能体定义来源于 SWM 同步至 MC 的内容，见 R-MC-014）与自动化脚本节点。本期干预切入点与策略匹配以人工为主，系统提供方案生成与编排支撑。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F38" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 舆情作战（作战编排）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G38" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-OCC-04 作战方案规划（作战参谋）；M-OCC-05 编排执行引擎（编排执行引擎）</x:t>
-        </x:is>
+      <x:c r="C38" s="3" t="str">
+        <x:v>行动编排</x:v>
+      </x:c>
+      <x:c r="D38" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
+      </x:c>
+      <x:c r="E38" s="3" t="str">
+        <x:v>根据目标档案与干预切入点匹配干预策略、生成作业方案，并以\"行动编排\"的方式直接编排群控子系统（MC）中的执行节点形成执行流程（图）落地，形成\"目标→编排→执行\"的闭环。OCC 直接编排 MC 中的节点，蜂群智能体子系统（SWM）作为\"智能体节点的供给方之一\"参与编排。编排的节点类型本期为两类——智能体节点（其智能体定义来源于 SWM 同步至 MC 的内容，见 R-MC-014）与自动化脚本节点。本期干预切入点与策略匹配以人工为主，系统提供方案生成与编排支撑。</x:v>
+      </x:c>
+      <x:c r="F38" s="3" t="str">
+        <x:v>需求.md 舆情行动（行动编排）</x:v>
+      </x:c>
+      <x:c r="G38" s="3" t="str">
+        <x:v>M-OCC-04 行动方案规划（行动参谋）；M-OCC-05 编排执行引擎（编排执行引擎）</x:v>
       </x:c>
       <x:c r="H38" s="3" t="inlineStr">
         <x:is>
           <x:t>F-OCC-04-01；F-OCC-04-02；F-OCC-05-01；F-OCC-05-02；F-OCC-05-03</x:t>
         </x:is>
       </x:c>
-      <x:c r="I38" s="3" t="inlineStr">
-        <x:is>
-          <x:t>II-10 作战编排下发与执行回传接口。</x:t>
-        </x:is>
+      <x:c r="I38" s="3" t="str">
+        <x:v>II-10 行动编排下发与执行回传接口。</x:v>
       </x:c>
       <x:c r="J38" s="3" t="inlineStr">
         <x:is>
@@ -3260,45 +3212,33 @@
           <x:t>效果评估</x:t>
         </x:is>
       </x:c>
-      <x:c r="D39" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>完成单轮干预成效统计、舆论走势修正、策略迭代反馈与作业复盘，并支持中短期与长期效果评估，形成作战闭环。本节的数据来源为两条：其一，数据爬取子系统（DC）的采集与分析结果（干预前后的舆情数据、传播数据、立场与情感变化）；其二，群控子系统（MC）可观测性能力（R-MC-010）上报的作业执行动作日志、任务日志与截图（投放触达、互动执行、账号行为记录）。OCC 基于这两类数据进行效果分析，不自行重复采集。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 舆情作战（效果评估）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-OCC-06 效果评估（作战复盘官）</x:t>
-        </x:is>
+      <x:c r="D39" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
+      </x:c>
+      <x:c r="E39" s="3" t="str">
+        <x:v>完成单轮干预成效统计、舆论走势修正、策略迭代反馈与作业复盘，并支持中短期与长期效果评估，形成行动闭环。本节的数据来源为两条：其一，数据爬取子系统（DC）的采集与分析结果（干预前后的舆情数据、传播数据、立场与情感变化）；其二，群控子系统（MC）可观测性能力（R-MC-010）上报的作业执行动作日志、任务日志与截图（投放触达、互动执行、账号行为记录）。OCC 基于这两类数据进行效果分析，不自行重复采集。</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>需求.md 舆情行动（效果评估）</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
+        <x:v>M-OCC-06 效果评估（行动复盘官）</x:v>
       </x:c>
       <x:c r="H39" s="3" t="inlineStr">
         <x:is>
           <x:t>F-OCC-06-01；F-OCC-06-02；F-OCC-06-03；F-OCC-06-04；F-OCC-06-05</x:t>
         </x:is>
       </x:c>
-      <x:c r="I39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，供 R-OCC-002~005 分析）、II-10 作战编排下发与执行回传（MC 作业数据来源）。</x:t>
-        </x:is>
+      <x:c r="I39" s="3" t="str">
+        <x:v>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，供 R-OCC-002~005 分析）、II-10 行动编排下发与执行回传（MC 作业数据来源）。</x:v>
       </x:c>
       <x:c r="J39" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试（效果评估与策略迭代反馈）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>可基于 DC 舆情数据与 MC 作业数据进行单轮干预成效统计（成效定义为可计算指标：投放触达率、互动率、目标群体立场/情感正向偏移量，均以干预前后 DC 采集数据差值量化）；可修正评估舆论走势（走势修正偏差以人工复核一致率不低于 80% 为达标）；可将评估反馈策略库迭代；可结合 MC 作业记录作业复盘；可提供中短期与长期效果评估接口（各项指标的具体达标线在详细设计阶段按作战类型细化）。</x:t>
-        </x:is>
+      <x:c r="K39" s="3" t="str">
+        <x:v>可基于 DC 舆情数据与 MC 作业数据进行单轮干预成效统计（成效定义为可计算指标：投放触达率、互动率、目标群体立场/情感正向偏移量，均以干预前后 DC 采集数据差值量化）；可修正评估舆论走势（走势修正偏差以人工复核一致率不低于 80% 为达标）；可将评估反馈策略库迭代；可结合 MC 作业记录作业复盘；可提供中短期与长期效果评估接口（各项指标的具体达标线在详细设计阶段按行动类型细化）。</x:v>
       </x:c>
       <x:c r="L39" s="6" t="inlineStr">
         <x:is>
@@ -3320,20 +3260,14 @@
           <x:t>舆论作业策略库</x:t>
         </x:is>
       </x:c>
-      <x:c r="D40" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E40" s="3" t="inlineStr">
-        <x:is>
-          <x:t>搭建并迭代多语种、多场景、多风格的舆论作业策略库，为作战提供可复用、可演进的策略资产。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F40" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 舆情作战（策略库）</x:t>
-        </x:is>
+      <x:c r="D40" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
+      </x:c>
+      <x:c r="E40" s="3" t="str">
+        <x:v>搭建并迭代多语种、多场景、多风格的舆论作业策略库，为行动提供可复用、可演进的策略资产。</x:v>
+      </x:c>
+      <x:c r="F40" s="3" t="str">
+        <x:v>需求.md 舆情行动（策略库）</x:v>
       </x:c>
       <x:c r="G40" s="3" t="inlineStr">
         <x:is>
@@ -3380,10 +3314,8 @@
           <x:t>内容资源管理</x:t>
         </x:is>
       </x:c>
-      <x:c r="D41" s="6" t="inlineStr">
-        <x:is>
-          <x:t>OCC 舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="D41" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E41" s="3" t="inlineStr">
         <x:is>
@@ -5553,10 +5485,8 @@
           <x:t>II-10</x:t>
         </x:is>
       </x:c>
-      <x:c r="D17" s="3" t="inlineStr">
-        <x:is>
-          <x:t>作战编排下发与执行回传</x:t>
-        </x:is>
+      <x:c r="D17" s="3" t="str">
+        <x:v>行动编排下发与执行回传</x:v>
       </x:c>
       <x:c r="E17" s="3" t="inlineStr">
         <x:is>
@@ -5658,10 +5588,8 @@
           <x:t>内容服务接口</x:t>
         </x:is>
       </x:c>
-      <x:c r="E19" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战 OCC</x:t>
-        </x:is>
+      <x:c r="E19" s="3" t="str">
+        <x:v>舆情行动 OCC</x:v>
       </x:c>
       <x:c r="F19" s="3" t="inlineStr">
         <x:is>
@@ -5763,10 +5691,8 @@
           <x:t>数据爬取 DC</x:t>
         </x:is>
       </x:c>
-      <x:c r="F21" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战 OCC</x:t>
-        </x:is>
+      <x:c r="F21" s="3" t="str">
+        <x:v>舆情行动 OCC</x:v>
       </x:c>
       <x:c r="G21" s="3" t="inlineStr">
         <x:is>
@@ -5950,9 +5876,6 @@
       <x:c r="B26" t="str">
         <x:v>内部接口 II</x:v>
       </x:c>
-      <x:c r="C26" t="str">
-        <x:v>II-18</x:v>
-      </x:c>
       <x:c r="D26" t="str">
         <x:v>用户画像查询接口</x:v>
       </x:c>
@@ -5982,17 +5905,17 @@
       <x:c r="B26" s="10" t="str">
         <x:v>内部接口 II</x:v>
       </x:c>
-      <x:c r="C26" s="10" t="str">
-        <x:v>II-17</x:v>
+      <x:c r="C26" t="str">
+        <x:v>II-18</x:v>
       </x:c>
       <x:c r="D26" s="11" t="str">
-        <x:v>COM 权限与组织管理接口</x:v>
+        <x:v>用户画像查询接口（V3.9 废止：ADR-001 删除，SWM R-SWM-005 改对话编写不再拉取画像）</x:v>
       </x:c>
       <x:c r="E26" s="11" t="str">
-        <x:v>公共功能 COM（M-COM-02）</x:v>
+        <x:v>舆情行动 OCC（已废）</x:v>
       </x:c>
       <x:c r="F26" s="11" t="str">
-        <x:v>各子系统 / 前端</x:v>
+        <x:v>蜂群 SWM（已废）</x:v>
       </x:c>
       <x:c r="G26" s="11" t="str">
         <x:v>入：用户/角色/组织配置；出：权限决策结果、组织结构。含用户/角色/组织 CRUD、账号解锁、RBAC 权限点查询。</x:v>
@@ -6191,10 +6114,8 @@
           <x:t>内容主数据（原始素材、分类、审核状态、来源）由 OCC 担任权威源统一维护</x:t>
         </x:is>
       </x:c>
-      <x:c r="E5" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战 OCC（权威源）</x:t>
-        </x:is>
+      <x:c r="E5" s="3" t="str">
+        <x:v>舆情行动 OCC（权威源）</x:v>
       </x:c>
       <x:c r="F5" s="3" t="inlineStr">
         <x:is>
@@ -6430,7 +6351,7 @@
         </x:is>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>蜂群智能体数据：以 agent_id（稳定逻辑标识）为索引的提示词包（人设标签、提示词、作业策略及当前生效版本号）及与 account_id 的 1:1 绑定关系、智能体作业记忆（Java 记忆服务 swm-memory 承载）与提示词模板版本</x:v>
+        <x:v>蜂群智能体数据：以 agent_id（稳定逻辑标识）为索引的提示词包（提示词、作业策略及当前生效版本号）及与 account_id 的 1:1 绑定关系、智能体作业记忆（Java 记忆服务 swm-memory 承载）与提示词模板版本</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
         <x:v>蜂群 SWM（提示词包生成/记忆承载）/群控 MC（提示词包持存）</x:v>
@@ -6488,25 +6409,17 @@
           <x:t>DR-11</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="6" t="inlineStr">
-        <x:is>
-          <x:t>业务数据-作战</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D14" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战数据：目标识别结果、传播链路、多维画像、抓手挖掘结果、作战编排流程（节点编排关系）、策略库版本与效果评估记录</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E14" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战 OCC</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F14" s="3" t="inlineStr">
-        <x:is>
-          <x:t>R-OCC-001~009（舆情作战数据）</x:t>
-        </x:is>
+      <x:c r="C14" s="6" t="str">
+        <x:v>业务数据-行动</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>舆情行动数据：目标识别结果、传播链路、多维画像、抓手挖掘结果、行动编排流程（节点编排关系）、策略库版本与效果评估记录</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>舆情行动 OCC</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>R-OCC-001~009（舆情行动数据）</x:v>
       </x:c>
       <x:c r="G14" s="6" t="inlineStr">
         <x:is>
@@ -6692,10 +6605,8 @@
           <x:t>阶段规划</x:t>
         </x:is>
       </x:c>
-      <x:c r="D5" s="3" t="inlineStr">
-        <x:is>
-          <x:t>蜂群智能体（SWM）、私有化大模型部署（IRS）、舆情作战（OCC）应优先实现核心闭环链路：本地大模型可用、蜂群可调度执行、舆情作战可形成识别到评估的闭环</x:t>
-        </x:is>
+      <x:c r="D5" s="3" t="str">
+        <x:v>蜂群智能体（SWM）、私有化大模型部署（IRS）、舆情行动（OCC）应优先实现核心闭环链路：本地大模型可用、蜂群可调度执行、舆情行动可形成识别到评估的闭环</x:v>
       </x:c>
       <x:c r="E5" s="3" t="inlineStr">
         <x:is>
@@ -6867,10 +6778,8 @@
           <x:t>架构约束</x:t>
         </x:is>
       </x:c>
-      <x:c r="D10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>执行终端应按指纹真实度进行风控分级，认知作战账号养号等高敏感场景应优先选用真机与 ARM 板卡，云手机与指纹浏览器 Profile 用于爬虫账号养护与规模化采集，模拟器仅用于测试</x:t>
-        </x:is>
+      <x:c r="D10" s="3" t="str">
+        <x:v>执行终端应按指纹真实度进行风控分级，认知行动账号养号等高敏感场景应优先选用真机与 ARM 板卡，云手机与指纹浏览器 Profile 用于爬虫账号养护与规模化采集，模拟器仅用于测试</x:v>
       </x:c>
       <x:c r="E10" s="3" t="inlineStr">
         <x:is>
@@ -6936,7 +6845,7 @@
         </x:is>
       </x:c>
       <x:c r="D12" s="3" t="str">
-        <x:v>执行层职责应按 统一执行网关 + 内容权威源 两类归属：指纹浏览器 Profile 的管理（创建、指纹固化、接入、监控）与桌面端 CDP 执行网关、移动端终端管理与 ADB/无障碍执行网关、账号主数据（注册、凭据、验证、风险评估、生命周期、账号分类）的唯一维护与共享分发、智能体执行宿主（含运行时 agent-runtime 子模块），均归群控子系统（MC）；内容资源（素材入库、分类、审核、排期、分发）唯一权威源归舆情作战业务子系统（OCC）。蜂群智能体子系统（SWM）作为提示词生成与记忆中心，将生成的提示词包（人设标签、提示词、作业策略）同步至 MC 持存，运行时（场景适配、动态调用、调用 IRS 推理）归 MC 的 agent-runtime 子模块；舆情作战子系统（OCC）以作战编排方式直接编排 MC 中的智能体节点与自动化脚本节点，使执行终端管理、账号主数据与动作执行统一收口</x:v>
+        <x:v>执行层职责应按 统一执行网关 + 内容权威源 两类归属：指纹浏览器 Profile 的管理（创建、指纹固化、接入、监控）与桌面端 CDP 执行网关、移动端终端管理与 ADB/无障碍执行网关、账号主数据（注册、凭据、验证、风险评估、生命周期、账号分类）的唯一维护与共享分发、智能体执行宿主（含运行时 agent-runtime 子模块），均归群控子系统（MC）；内容资源（素材入库、分类、审核、排期、分发）唯一权威源归舆情行动业务子系统（OCC）。蜂群智能体子系统（SWM）作为提示词生成与记忆中心，将生成的提示词包（提示词、作业策略）同步至 MC 持存，运行时（场景适配、动态调用、调用 IRS 推理）归 MC 的 agent-runtime 子模块；舆情行动子系统（OCC）以行动编排方式直接编排 MC 中的智能体节点与自动化脚本节点，使执行终端管理、账号主数据与动作执行统一收口</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
         <x:v>R-MC-001/005/006/011/014；R-OCC-009（执行层职责归属）</x:v>
@@ -7001,10 +6910,8 @@
           <x:t>架构约束</x:t>
         </x:is>
       </x:c>
-      <x:c r="D14" s="3" t="inlineStr">
-        <x:is>
-          <x:t>账号应按用途分类管理：爬虫账号以桌面端指纹浏览器 Profile 为执行终端、其养护（养号）动作执行经 MC 统一执行网关的 CDP 通道，认知作战账号以移动端设备为执行终端、经 MC 统一执行网关的 ADB/无障碍通道执行养号动作；两类账号的注册、验证与生命周期等主数据均由群控子系统（MC）统一维护并向各子系统分发 account_id。账号-终端-代理绑定遵循差异化规则：真机、云手机、虚拟化真机执行"一设备一账号一 IP"，指纹浏览器 Profile 执行"一 Profile 一账号一 IP"（实例可多开），每个终端/Profile 绑定一个固定代理 IP</x:t>
-        </x:is>
+      <x:c r="D14" s="3" t="str">
+        <x:v>账号应按用途分类管理：爬虫账号以桌面端指纹浏览器 Profile 为执行终端、其养护（养号）动作执行经 MC 统一执行网关的 CDP 通道，认知行动账号以移动端设备为执行终端、经 MC 统一执行网关的 ADB/无障碍通道执行养号动作；两类账号的注册、验证与生命周期等主数据均由群控子系统（MC）统一维护并向各子系统分发 account_id。账号-终端-代理绑定遵循差异化规则：真机、云手机、虚拟化真机执行\</x:v>
       </x:c>
       <x:c r="E14" s="3" t="inlineStr">
         <x:is>
@@ -7330,10 +7237,8 @@
           <x:t>OCC</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>舆情作战业务子系统</x:t>
-        </x:is>
+      <x:c r="B10" s="3" t="str">
+        <x:v>舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="C10" s="6" t="n">
         <x:v>9</x:v>

</xml_diff>

<commit_message>
vault backup: 2026-07-20 21:04:43
</commit_message>
<xml_diff>
--- a/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
+++ b/公司项目/认知作战/文档/软件需求跟踪矩阵.xlsx
@@ -16,7 +16,7 @@
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="追溯汇总统计" sheetId="7" state="visible" r:id="rId7"/>
   </x:sheets>
   <x:definedNames>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'功能需求跟踪矩阵'!$A$1:$L$41</x:definedName>
+    <x:definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'功能需求跟踪矩阵'!$A$1:$L$42</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'非功能需求跟踪矩阵'!$A$1:$G$36</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'接口需求跟踪矩阵'!$A$1:$J$23</x:definedName>
     <x:definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'数据需求跟踪矩阵'!$A$1:$G$14</x:definedName>
@@ -1603,10 +1603,8 @@
           <x:t>F-MC-01-01；F-MC-01-02；F-MC-01-03；F-MC-01-04</x:t>
         </x:is>
       </x:c>
-      <x:c r="I10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>EI-04 对象存储、EI-06 指纹浏览器服务、II-02 Agent 指令与日志、II-04 日志指标上报（至 OM）。</x:t>
-        </x:is>
+      <x:c r="I10" s="3" t="str">
+        <x:v>EI-04 对象存储、EI-06 指纹浏览器服务、II-04 日志指标上报（至 OM）、R-MC-015 设备上下线事件订阅（内部，V4.1 / V3.10 改）。</x:v>
       </x:c>
       <x:c r="J10" s="3" t="inlineStr">
         <x:is>
@@ -1963,10 +1961,8 @@
           <x:t>F-MC-07-01；F-MC-07-02；F-MC-07-03；F-MC-07-04；F-MC-07-05</x:t>
         </x:is>
       </x:c>
-      <x:c r="I16" s="3" t="inlineStr">
-        <x:is>
-          <x:t>II-02 Agent 指令与日志、II-04 日志指标上报（至 OM）。</x:t>
-        </x:is>
+      <x:c r="I16" s="3" t="str">
+        <x:v>II-02 Agent 长连接协议（V4.1 / V3.10 提供方调整为 R-MC-015，本需求订阅其事件）、II-04 日志指标上报（至 OM）。</x:v>
       </x:c>
       <x:c r="J16" s="3" t="inlineStr">
         <x:is>
@@ -2385,372 +2381,354 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="6" t="n">
+      <x:c r="A24">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="B24" s="6" t="inlineStr">
+      <x:c r="B24" t="str">
+        <x:v>R-MC-015</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>真机 Agent 运行时与编排</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>MC 多设备矩阵自动化群控子系统</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>提供真机 Agent 运行时（设备主机侧独立部署单元）+ 中心侧 Agent 编排网关，承载真机设备的连接生命周期（注册/心跳/占用锁）、真机控制通道（ADB/无障碍）、远控画面源（scrcpy H.264 喂 mc-sfu）。Agent 是 MC 体系内唯一触碰真机的进程（CON-15）；所有真机动作经 R-MC-005 统一执行网关收口，由网关路由到本需求实现的 RealDeviceSdk，再经 II-02 长连接下发 Agent 落地。V4.1 / V3.10 新增，借鉴 SonicCloudOrg（已 archived，Apache 2.0 fork 自维护）。</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>SRS V4.1 MC 分册 R-MC-015；SonicCloudOrg sonic-agent 架构借鉴</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>M-MC-15 真机 Agent 运行时与编排（双形态：M-MC-15.c 中心侧编排器 + M-MC-15.a 设备主机侧 Agent 运行时）</x:v>
+      </x:c>
+      <x:c r="H24" t="str">
+        <x:v>F-MC-15-01；F-MC-15-02；F-MC-15-03；F-MC-15-04；F-MC-15-05；F-MC-15-06</x:v>
+      </x:c>
+      <x:c r="I24" t="str">
+        <x:v>II-02 Agent 长连接协议（本需求为提供方）、II-03 远控画面传输（与 R-MC-004 协商）、II-07 执行网关动作接口（本需求为 RealDeviceSdk 实现方）。</x:v>
+      </x:c>
+      <x:c r="J24" t="str">
+        <x:v>功能测试 + 演示（Agent 注册/心跳/占用、ADB/无障碍动作落地、scrcpy 远控画面源）</x:v>
+      </x:c>
+      <x:c r="K24" t="str">
+        <x:v>Agent 启动可经 II-02 连中心侧编排器并完成鉴权与设备清单上报；Agent 心跳可被识别并维护在线状态、超时可判离线并通知台账；真机动作经网关可路由到本模块、经 II-02 下发 Agent 落地（ADB install/pressKey/reboot/screenshot 与无障碍 find/click/sendKeys/swipe）；远控打开时 Agent 可启动 scrcpy 推流到 mc-sfu、浏览器经 mc-sfu WebRTC 看到画面；占用锁可保证同一台设备同时只有一个会话使用；Agent 断线可自动重连。</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>✓ 完整</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="6">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B25" s="6" t="inlineStr">
         <x:is>
           <x:t>R-OM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="C24" s="3" t="inlineStr">
+      <x:c r="C25" s="3" t="inlineStr">
         <x:is>
           <x:t>日志与指标汇聚</x:t>
         </x:is>
       </x:c>
-      <x:c r="D24" s="6" t="inlineStr">
+      <x:c r="D25" s="6" t="inlineStr">
         <x:is>
           <x:t>OM 运维监控子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E24" s="3" t="inlineStr">
+      <x:c r="E25" s="3" t="inlineStr">
         <x:is>
           <x:t>汇聚数据爬取子系统、群控子系统及平台自身的日志与指标，形成统一的运维数据底座，支撑全系统可观测。</x:t>
         </x:is>
       </x:c>
-      <x:c r="F24" s="3" t="inlineStr">
+      <x:c r="F25" s="3" t="inlineStr">
         <x:is>
           <x:t>需求.md 运维监控（日志与指标汇聚）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G24" s="3" t="inlineStr">
+      <x:c r="G25" s="3" t="inlineStr">
         <x:is>
           <x:t>M-OM-01 日志汇聚与检索（日志数据底座）；M-OM-02 指标采集与时序存储（指标数据底座）</x:t>
         </x:is>
       </x:c>
-      <x:c r="H24" s="3" t="inlineStr">
+      <x:c r="H25" s="3" t="inlineStr">
         <x:is>
           <x:t>F-OM-01-01；F-OM-01-02；F-OM-02-01；F-OM-02-02</x:t>
         </x:is>
       </x:c>
-      <x:c r="I24" s="3" t="inlineStr">
+      <x:c r="I25" s="3" t="inlineStr">
         <x:is>
           <x:t>II-04 日志与指标上报接口。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J24" s="3" t="str">
+      <x:c r="J25" s="3" t="str">
         <x:v>功能测试 + 演示（复用 KubeSphere 可观测底座，OM 只读查询代理 + 分析入仓；详见 OM SDD §5.1/§5.2/§6）</x:v>
       </x:c>
-      <x:c r="K24" s="3" t="inlineStr">
+      <x:c r="K25" s="3" t="inlineStr">
         <x:is>
           <x:t>各子系统日志可汇聚至统一日志库并支持全文检索；关键指标可采集为时序数据；近 7 日日志检索响应不大于 3 秒。</x:t>
         </x:is>
       </x:c>
-      <x:c r="L24" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="6" t="n">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B25" s="6" t="inlineStr">
+      <x:c r="L25" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="6">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="B26" s="6" t="inlineStr">
         <x:is>
           <x:t>R-OM-002</x:t>
         </x:is>
       </x:c>
-      <x:c r="C25" s="3" t="inlineStr">
+      <x:c r="C26" s="3" t="inlineStr">
         <x:is>
           <x:t>告警与运维</x:t>
         </x:is>
       </x:c>
-      <x:c r="D25" s="6" t="inlineStr">
+      <x:c r="D26" s="6" t="inlineStr">
         <x:is>
           <x:t>OM 运维监控子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E25" s="3" t="inlineStr">
+      <x:c r="E26" s="3" t="inlineStr">
         <x:is>
           <x:t>基于指标与规则产生告警，并通过仪表盘与运维操作支持常态化运维。</x:t>
         </x:is>
       </x:c>
-      <x:c r="F25" s="3" t="inlineStr">
+      <x:c r="F26" s="3" t="inlineStr">
         <x:is>
           <x:t>需求.md 运维监控（告警与运维）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G25" s="3" t="str">
+      <x:c r="G26" s="3" t="str">
         <x:v>M-OM-03 告警引擎（告警观测，只读观测 Alertmanager 规则/事件 + 事件归档）；M-OM-04 运维可视化与作业（运维作业台）</x:v>
       </x:c>
-      <x:c r="H25" s="3" t="inlineStr">
+      <x:c r="H26" s="3" t="inlineStr">
         <x:is>
           <x:t>F-OM-03-01；F-OM-03-02；F-OM-04-01；F-OM-04-02</x:t>
         </x:is>
       </x:c>
-      <x:c r="I25" s="3" t="inlineStr">
+      <x:c r="I26" s="3" t="inlineStr">
         <x:is>
           <x:t>无（依赖 R-OM-001 时序指标数据）。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J25" s="3" t="str">
+      <x:c r="J26" s="3" t="str">
         <x:v>功能测试 + 演示（告警规则配置由 KubeSphere 控制台承担，OM 只读观测；详见 OM SDD §5.3/§6）</x:v>
       </x:c>
-      <x:c r="K25" s="3" t="inlineStr">
+      <x:c r="K26" s="3" t="inlineStr">
         <x:is>
           <x:t>阈值与异常检测告警可触发并多渠道通知；多维看板可可视化展示；日志查询、故障定位、巡检、容量观测等运维操作可执行。</x:t>
         </x:is>
       </x:c>
-      <x:c r="L25" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="6" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="B26" s="6" t="inlineStr">
+      <x:c r="L26" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="6">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B27" s="6" t="inlineStr">
         <x:is>
           <x:t>R-COM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="C26" s="3" t="inlineStr">
+      <x:c r="C27" s="3" t="inlineStr">
         <x:is>
           <x:t>用户认证与权限</x:t>
         </x:is>
       </x:c>
-      <x:c r="D26" s="6" t="inlineStr">
+      <x:c r="D27" s="6" t="inlineStr">
         <x:is>
           <x:t>COM 公共功能</x:t>
         </x:is>
       </x:c>
-      <x:c r="E26" s="3" t="inlineStr">
+      <x:c r="E27" s="3" t="inlineStr">
         <x:is>
           <x:t>用户认证与权限</x:t>
         </x:is>
       </x:c>
-      <x:c r="F26" s="3" t="inlineStr">
+      <x:c r="F27" s="3" t="inlineStr">
         <x:is>
           <x:t>开发方案 V1.1 安全设计（认证授权）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G26" s="3" t="inlineStr">
+      <x:c r="G27" s="3" t="inlineStr">
         <x:is>
           <x:t>M-COM-01 身份认证（身份守门人）；M-COM-02 权限与组织管理（权限决策与组织隔离）</x:t>
         </x:is>
       </x:c>
-      <x:c r="H26" s="3" t="str">
+      <x:c r="H27" s="3" t="str">
         <x:v>F-COM-01-01；F-COM-01-03；F-COM-02-01；F-COM-02-02；F-COM-02-03</x:v>
       </x:c>
-      <x:c r="I26" s="3" t="str">
+      <x:c r="I27" s="3" t="str">
         <x:v>II-16 COM 认证服务（M-COM-01）；II-17 COM 权限与组织管理（M-COM-02）；各子系统统一调用。</x:v>
       </x:c>
-      <x:c r="J26" s="3" t="inlineStr">
+      <x:c r="J27" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试（认证授权、多组织隔离）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K26" s="3" t="str">
+      <x:c r="K27" s="3" t="str">
         <x:v>登录认证可用；RBAC 权限决策可按角色控制；多组织数据可隔离且禁止跨组织访问。</x:v>
       </x:c>
-      <x:c r="L26" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="6" t="n">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B27" s="6" t="inlineStr">
+      <x:c r="L27" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="6">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="B28" s="6" t="inlineStr">
         <x:is>
           <x:t>R-SWM-001</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" s="3" t="str">
+      <x:c r="C28" s="3" t="str">
         <x:v>提示词管理</x:v>
       </x:c>
-      <x:c r="D27" s="6" t="inlineStr">
+      <x:c r="D28" s="6" t="inlineStr">
         <x:is>
           <x:t>SWM 蜂群智能体子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E27" s="3" t="str">
+      <x:c r="E28" s="3" t="str">
         <x:v>管理驱动智能体作业的提示词，支持提示词模板库分类、版本管理、Playground 试运行调试、版本输出对比与迭代优化，并以 agent_id（模板共性）+ account_id（动态实例个性）组合为标识将提示词包（提示词模板、账号级动态提示词实例、作业策略）同步至 MC 持存。V3.9（ADR-001）废除人设标签实体，人设属性直接写进提示词文本。账号主数据由 MC 统一维护（R-MC-011）。运行时场景适配与动态调用归 MC 的 agent-runtime 子模块（见 R-MC-006/014）。</x:v>
       </x:c>
-      <x:c r="F27" s="3" t="inlineStr">
+      <x:c r="F28" s="3" t="inlineStr">
         <x:is>
           <x:t>需求.md 蜂群智能体（提示词与人设管理）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G27" s="3" t="str">
+      <x:c r="G28" s="3" t="str">
         <x:v>M-SWM-01 提示词管理（V3.9 改：原人设标签管理废除，改提示词模板/版本管理）；M-SWM-02 提示词模板库与版本管理（提示词资产管理）</x:v>
       </x:c>
-      <x:c r="H27" s="3" t="str">
+      <x:c r="H28" s="3" t="str">
         <x:v>F-SWM-01-01；F-SWM-01-02；F-SWM-02-01；F-SWM-02-02；F-SWM-02-03；F-SWM-02-04</x:v>
       </x:c>
-      <x:c r="I27" s="3" t="str">
+      <x:c r="I28" s="3" t="str">
         <x:v>EI-05 本地大模型推理（Playground 试运行与版本对比推理）、II-14 提示词包同步接口。</x:v>
       </x:c>
-      <x:c r="J27" s="3" t="str">
+      <x:c r="J28" s="3" t="str">
         <x:v>功能测试（人设绑 agent_id、模板库、版本/Playground/对比）</x:v>
       </x:c>
-      <x:c r="K27" s="3" t="str">
+      <x:c r="K28" s="3" t="str">
         <x:v>提示词模板库可分类管理；版本可按 agent_id 对比回滚（账号级动态实例按 account_id）；可在 Playground 中填入提示词草稿即时调用 IRS 试运行并查看产出；可将不同版本提示词并排对比输出；可结合反馈与调优结果迭代优化；提示词包可以 agent_id+account_id 组合同步至 MC 持存。</x:v>
       </x:c>
-      <x:c r="L27" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="6" t="n">
-        <x:v>27</x:v>
-      </x:c>
-      <x:c r="B28" s="6" t="inlineStr">
+      <x:c r="L28" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="6">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="B29" s="6" t="inlineStr">
         <x:is>
           <x:t>R-SWM-002</x:t>
         </x:is>
       </x:c>
-      <x:c r="C28" s="3" t="inlineStr">
+      <x:c r="C29" s="3" t="inlineStr">
         <x:is>
           <x:t>蜂群记忆管理</x:t>
         </x:is>
       </x:c>
-      <x:c r="D28" s="6" t="inlineStr">
+      <x:c r="D29" s="6" t="inlineStr">
         <x:is>
           <x:t>SWM 蜂群智能体子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E28" s="3" t="str">
+      <x:c r="E29" s="3" t="str">
         <x:v>实现智能体作业记忆的存储、场景沉淀、历史复用与个性化状态延续，使智能体长期行为符合人设且不断演进。记忆按 account_id 1:1 归属（账号级独立，同一 agent 下不同账号各自独立记忆）。</x:v>
       </x:c>
-      <x:c r="F28" s="3" t="inlineStr">
+      <x:c r="F29" s="3" t="inlineStr">
         <x:is>
           <x:t>需求.md 蜂群智能体（记忆管理）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G28" s="3" t="inlineStr">
+      <x:c r="G29" s="3" t="inlineStr">
         <x:is>
           <x:t>M-SWM-04 蜂群记忆管理（智能体记忆中枢）</x:t>
         </x:is>
       </x:c>
-      <x:c r="H28" s="3" t="inlineStr">
+      <x:c r="H29" s="3" t="inlineStr">
         <x:is>
           <x:t>F-SWM-04-01；F-SWM-04-02；F-SWM-04-03；F-SWM-04-04</x:t>
         </x:is>
       </x:c>
-      <x:c r="I28" s="3" t="str">
+      <x:c r="I29" s="3" t="str">
         <x:v>无（记忆为 SWM 内部存储，载体为 Java 记忆服务 swm-memory）。</x:v>
       </x:c>
-      <x:c r="J28" s="3" t="inlineStr">
+      <x:c r="J29" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试（记忆存储/沉淀/复用/延续）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K28" s="3" t="str">
+      <x:c r="K29" s="3" t="str">
         <x:v>作业关键信息可按 account_id 记忆存储（账号级 1:1 归属）；重复场景经验可沉淀为模式；相似作业可复用历史记忆；智能体可基于账号级记忆维持个性化延续；启用记忆后智能体的人设一致性有效性由评测子系统（R-SWM-004）的 loop 评估器度量，人设一致性评分须达到 loop 评估器设定的可用线，且跨轮次作业的行为连贯性不退化。</x:v>
       </x:c>
-      <x:c r="L28" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="6" t="n">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B29" s="6" t="inlineStr">
+      <x:c r="L29" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="6">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B30" s="6" t="inlineStr">
         <x:is>
           <x:t>R-SWM-003</x:t>
         </x:is>
       </x:c>
-      <x:c r="C29" s="3" t="inlineStr">
+      <x:c r="C30" s="3" t="inlineStr">
         <x:is>
           <x:t>智能体构建</x:t>
         </x:is>
       </x:c>
-      <x:c r="D29" s="6" t="inlineStr">
+      <x:c r="D30" s="6" t="inlineStr">
         <x:is>
           <x:t>SWM 蜂群智能体子系统</x:t>
         </x:is>
       </x:c>
-      <x:c r="E29" s="3" t="str">
+      <x:c r="E30" s="3" t="str">
         <x:v>根据提示词（画像、账号属性）构建可作业的智能体——配置驱动作业的提示词模板与作业策略（目标、场景、边界），组装为提示词包（提示词模板、账号级动态提示词实例、作业策略）并以 agent_id（模板共性，稳定逻辑标识）+ account_id（动态实例个性）组合为标识，经内部接口 II-14 同步至群控子系统（MC）持存、供舆情行动子系统（OCC）行动编排引用。记忆不在提示词包内，由记忆服务（account_id 主键）独立承载。本功能确立 SWM 生成提示词包、MC 持存并运行（agent-runtime）、OCC 编排引用 的分工。</x:v>
       </x:c>
-      <x:c r="F29" s="3" t="inlineStr">
+      <x:c r="F30" s="3" t="inlineStr">
         <x:is>
           <x:t>需求.md 蜂群智能体（智能体构建）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G29" s="3" t="str">
+      <x:c r="G30" s="3" t="str">
         <x:v>M-SWM-05 智能体构建与提示词包下发（智能体装配工厂）</x:v>
       </x:c>
-      <x:c r="H29" s="3" t="str">
+      <x:c r="H30" s="3" t="str">
         <x:v>F-SWM-05-01；F-SWM-05-02；F-SWM-05-03；F-SWM-05-04</x:v>
       </x:c>
-      <x:c r="I29" s="3" t="str">
+      <x:c r="I30" s="3" t="str">
         <x:v>II-01 账号服务接口、II-14 提示词包同步接口。</x:v>
       </x:c>
-      <x:c r="J29" s="3" t="inlineStr">
+      <x:c r="J30" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试 + 演示（构建/1:1 绑定/同步/节点来源）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K29" s="3" t="str">
+      <x:c r="K30" s="3" t="str">
         <x:v>可按提示词构建提示词包并以 agent_id（模板）+ account_id（动态实例）组合为标识；提示词包须包含提示词模板、作业策略必填要素，缺一不可构建；agent_id 为稳定逻辑标识、提示词模板版本可随重生成升级；可与 account_id 1:N 绑定（一个 agent 绑多个账号，每账号独立动态实例）；提示词包可经 II-14 以 agent_id+account_id 组合同步至 MC 持存并取得版本号且同步成功率不低于 99%；构建出的智能体可作为 OCC 行动编排的智能体节点来源。</x:v>
-      </x:c>
-      <x:c r="L29" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="6" t="n">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="B30" s="6" t="inlineStr">
-        <x:is>
-          <x:t>R-SWM-004</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>智能体评测</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D30" s="6" t="inlineStr">
-        <x:is>
-          <x:t>SWM 蜂群智能体子系统</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E30" s="3" t="str">
-        <x:v>对构建出的智能体（R-SWM-003）进行质量评测，采用「线上效果 + 离线数据集」双轨评测范式评估智能体的有效性、稳定性与合规性；离线评测以"评测集、评估器、实验"三类可管理实体组织——评测集承载测试用例，评估器承载可复用的打分逻辑，实验承载一次可追踪、可对比的评测运行，淘汰低效定义、迭代优化高价值定义，形成"构建→评测→迭代"的闭环，使智能体定义随作业实践持续演进。双轨评测互补印证：线上效果反映真实行动表现，离线数据集提供受控、可复现、可对比的质量基准，避免单一维度误判。</x:v>
-      </x:c>
-      <x:c r="F30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 蜂群智能体（智能体评测）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-SWM-06 智能体评测与迭代决策（智能体质量裁判）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>F-SWM-06-01；F-SWM-06-02；F-SWM-06-03；F-SWM-06-04；F-SWM-06-05；F-SWM-06-06</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I30" s="3" t="str">
-        <x:v>EI-05 本地大模型推理（离线跑题）、II-10 行动编排下发与执行回传（MC 作业效果数据来源）。</x:v>
-      </x:c>
-      <x:c r="J30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>功能测试（双轨评测、迭代/淘汰决策）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K30" s="3" t="inlineStr">
-        <x:is>
-          <x:t>可基于 MC 作业效果数据评测智能体线上有效性；可基于标准评测数据集完成离线跑题、答案对比打分与评分汇总；可创建/编辑/版本化评估器并跨实验引用；可发起实验并持久化记录其输入快照、逐题结果、各维度评分与运行状态；可对同一数据集多次发起实验并横向对比版本演进；可产出各维度评分与迭代/淘汰决策并反馈至 R-SWM-001 与 R-SWM-003 形成闭环。离线评测各维度采用百分制，及格线 60 分、淘汰线 40 分（低于 40 分直接淘汰、40~60 分进入迭代优化、60 分以上为可用），线上有效性评测的任务完成率低于 50% 触发迭代（具体门槛在详细设计阶段按作业类型细化）。</x:t>
-        </x:is>
       </x:c>
       <x:c r="L30" s="6" t="inlineStr">
         <x:is>
@@ -2762,98 +2740,94 @@
       <x:c r="A31" s="6">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="B31" s="6" t="str">
-        <x:v>R-SWM-005</x:v>
-      </x:c>
-      <x:c r="C31" s="3" t="str">
-        <x:v>对话编写提示词</x:v>
-      </x:c>
-      <x:c r="D31" s="6" t="str">
-        <x:v>SWM 蜂群智能体子系统</x:v>
+      <x:c r="B31" s="6" t="inlineStr">
+        <x:is>
+          <x:t>R-SWM-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>智能体评测</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D31" s="6" t="inlineStr">
+        <x:is>
+          <x:t>SWM 蜂群智能体子系统</x:t>
+        </x:is>
       </x:c>
       <x:c r="E31" s="3" t="str">
-        <x:v>用户上传画像素材或描述需求，经 IRS 本地大模型对话式辅助编写提示词（V3.9 改：ADR-001，不再经 II-01/II-18 系统拉取）；生成结果纳入版本管理并可作为 R-SWM-003 智能体构建的提示词来源。</x:v>
-      </x:c>
-      <x:c r="F31" s="3" t="str">
-        <x:v>需求.md 蜂群智能体（提示词自动生成）</x:v>
-      </x:c>
-      <x:c r="G31" s="3" t="str">
-        <x:v>M-SWM-07 对话编写提示词（对话编写引擎）</x:v>
-      </x:c>
-      <x:c r="H31" s="3" t="str">
-        <x:v>F-SWM-07-01；F-SWM-07-02；F-SWM-07-03</x:v>
+        <x:v>对构建出的智能体（R-SWM-003）进行质量评测，采用「线上效果 + 离线数据集」双轨评测范式评估智能体的有效性、稳定性与合规性；离线评测以"评测集、评估器、实验"三类可管理实体组织——评测集承载测试用例，评估器承载可复用的打分逻辑，实验承载一次可追踪、可对比的评测运行，淘汰低效定义、迭代优化高价值定义，形成"构建→评测→迭代"的闭环，使智能体定义随作业实践持续演进。双轨评测互补印证：线上效果反映真实行动表现，离线数据集提供受控、可复现、可对比的质量基准，避免单一维度误判。</x:v>
+      </x:c>
+      <x:c r="F31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>需求.md 蜂群智能体（智能体评测）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>M-SWM-06 智能体评测与迭代决策（智能体质量裁判）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>F-SWM-06-01；F-SWM-06-02；F-SWM-06-03；F-SWM-06-04；F-SWM-06-05；F-SWM-06-06</x:t>
+        </x:is>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>EI-05 本地大模型推理（对话编写推理）。V3.9 删 II-01/II-18（不再系统拉取）。</x:v>
-      </x:c>
-      <x:c r="J31" s="3" t="str">
-        <x:v>功能测试（素材上传、对话编写、IRS 推理、版本化纳入构建）</x:v>
-      </x:c>
-      <x:c r="K31" s="3" t="str">
-        <x:v>可上传画像素材并描述需求；可与 IRS 对话式编写提示词；生成结果可版本化并回写提示词库；可经人工审核微调后纳入 R-SWM-003 智能体构建。</x:v>
-      </x:c>
-      <x:c r="L31" s="6" t="str">
-        <x:v>✓ 完整</x:v>
+        <x:v>EI-05 本地大模型推理（离线跑题）、II-10 行动编排下发与执行回传（MC 作业效果数据来源）。</x:v>
+      </x:c>
+      <x:c r="J31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>功能测试（双轨评测、迭代/淘汰决策）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K31" s="3" t="inlineStr">
+        <x:is>
+          <x:t>可基于 MC 作业效果数据评测智能体线上有效性；可基于标准评测数据集完成离线跑题、答案对比打分与评分汇总；可创建/编辑/版本化评估器并跨实验引用；可发起实验并持久化记录其输入快照、逐题结果、各维度评分与运行状态；可对同一数据集多次发起实验并横向对比版本演进；可产出各维度评分与迭代/淘汰决策并反馈至 R-SWM-001 与 R-SWM-003 形成闭环。离线评测各维度采用百分制，及格线 60 分、淘汰线 40 分（低于 40 分直接淘汰、40~60 分进入迭代优化、60 分以上为可用），线上有效性评测的任务完成率低于 50% 触发迭代（具体门槛在详细设计阶段按作业类型细化）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L31" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="6">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="B32" s="6" t="inlineStr">
-        <x:is>
-          <x:t>R-IRS-001</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>本地大模型部署</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D32" s="6" t="inlineStr">
-        <x:is>
-          <x:t>IRS 私有化大模型部署</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>在私有化环境中部署本地大模型，构建系统的底座推理能力，使全系统的 AI 推理不依赖外部公有云，供各子系统统一调用。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 私有化推理（本地大模型部署）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-IRS-01 本地大模型部署（底座推理能力提供者）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>F-IRS-01-01；F-IRS-01-02；F-IRS-01-03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>EI-05 本地大模型推理接口。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>功能测试（私有化部署与推理调用）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K32" s="3" t="inlineStr">
-        <x:is>
-          <x:t>本地大模型可在私有化环境部署并加载实例化；可对外提供推理调用接口；部署不依赖外部公有云。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L32" s="6" t="inlineStr">
-        <x:is>
-          <x:t>✓ 完整</x:t>
-        </x:is>
+      <x:c r="B32" s="6" t="str">
+        <x:v>R-SWM-005</x:v>
+      </x:c>
+      <x:c r="C32" s="3" t="str">
+        <x:v>对话编写提示词</x:v>
+      </x:c>
+      <x:c r="D32" s="6" t="str">
+        <x:v>SWM 蜂群智能体子系统</x:v>
+      </x:c>
+      <x:c r="E32" s="3" t="str">
+        <x:v>用户上传画像素材或描述需求，经 IRS 本地大模型对话式辅助编写提示词（V3.9 改：ADR-001，不再经 II-01/II-18 系统拉取）；生成结果纳入版本管理并可作为 R-SWM-003 智能体构建的提示词来源。</x:v>
+      </x:c>
+      <x:c r="F32" s="3" t="str">
+        <x:v>需求.md 蜂群智能体（提示词自动生成）</x:v>
+      </x:c>
+      <x:c r="G32" s="3" t="str">
+        <x:v>M-SWM-07 对话编写提示词（对话编写引擎）</x:v>
+      </x:c>
+      <x:c r="H32" s="3" t="str">
+        <x:v>F-SWM-07-01；F-SWM-07-02；F-SWM-07-03</x:v>
+      </x:c>
+      <x:c r="I32" s="3" t="str">
+        <x:v>EI-05 本地大模型推理（对话编写推理）。V3.9 删 II-01/II-18（不再系统拉取）。</x:v>
+      </x:c>
+      <x:c r="J32" s="3" t="str">
+        <x:v>功能测试（素材上传、对话编写、IRS 推理、版本化纳入构建）</x:v>
+      </x:c>
+      <x:c r="K32" s="3" t="str">
+        <x:v>可上传画像素材并描述需求；可与 IRS 对话式编写提示词；生成结果可版本化并回写提示词库；可经人工审核微调后纳入 R-SWM-003 智能体构建。</x:v>
+      </x:c>
+      <x:c r="L32" s="6" t="str">
+        <x:v>✓ 完整</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2862,46 +2836,52 @@
       </x:c>
       <x:c r="B33" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-001</x:t>
+          <x:t>R-IRS-001</x:t>
         </x:is>
       </x:c>
       <x:c r="C33" s="3" t="inlineStr">
         <x:is>
-          <x:t>目标识别与维护</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D33" s="6" t="str">
-        <x:v>OCC 舆情行动业务子系统</x:v>
-      </x:c>
-      <x:c r="E33" s="3" t="str">
-        <x:v>识别舆情事件的目标要素并对其进行全生命周期维护。目标在系统中即数据对象——支持建档、修改、关联、状态流转与删除，而非一次识别即定型的只读结果。本能力融合情报侦察、多维画像与抓手挖掘中\"识别目标\"的部分：从舆情事件与传播数据中识别事件主体、传播源头、核心争议点、干预目标对象，并补充传播线索、事件/群体/账号/传播画像、干预切入点与薄弱点等目标属性，形成可持续维护的目标档案，为后续行动提供靶向。</x:v>
-      </x:c>
-      <x:c r="F33" s="3" t="str">
-        <x:v>需求.md 舆情行动（目标识别与维护）</x:v>
+          <x:t>本地大模型部署</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="6" t="inlineStr">
+        <x:is>
+          <x:t>IRS 私有化大模型部署</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E33" s="3" t="inlineStr">
+        <x:is>
+          <x:t>在私有化环境中部署本地大模型，构建系统的底座推理能力，使全系统的 AI 推理不依赖外部公有云，供各子系统统一调用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F33" s="3" t="inlineStr">
+        <x:is>
+          <x:t>需求.md 私有化推理（本地大模型部署）</x:t>
+        </x:is>
       </x:c>
       <x:c r="G33" s="3" t="inlineStr">
         <x:is>
-          <x:t>M-OCC-01 目标档案与状态管理（目标数据管家）；M-OCC-03 目标关联网络（目标关系图谱）</x:t>
+          <x:t>M-IRS-01 本地大模型部署（底座推理能力提供者）</x:t>
         </x:is>
       </x:c>
       <x:c r="H33" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-01-01；F-OCC-01-02；F-OCC-01-03；F-OCC-01-04；F-OCC-01-05；F-OCC-03-01；F-OCC-03-02</x:t>
+          <x:t>F-IRS-01-01；F-IRS-01-02；F-IRS-01-03</x:t>
         </x:is>
       </x:c>
       <x:c r="I33" s="3" t="inlineStr">
         <x:is>
-          <x:t>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，经 R-OCC-002~005 分析后供目标识别融合）、EI-05 本地大模型推理（辅助识别）。</x:t>
+          <x:t>EI-05 本地大模型推理接口。</x:t>
         </x:is>
       </x:c>
       <x:c r="J33" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（建档/修改/关联/状态流转）</x:t>
+          <x:t>功能测试（私有化部署与推理调用）</x:t>
         </x:is>
       </x:c>
       <x:c r="K33" s="3" t="inlineStr">
         <x:is>
-          <x:t>目标可建档并赋予 target_id；目标各属性可新增、修改、删除；目标间可建立关联关系；目标状态可流转；目标档案可融合事件主体、传播、画像、切入点等多维信息；目标变更可经事件通知使用方；本期支持人工识别录入与系统数据维护。</x:t>
+          <x:t>本地大模型可在私有化环境部署并加载实例化；可对外提供推理调用接口；部署不依赖外部公有云。</x:t>
         </x:is>
       </x:c>
       <x:c r="L33" s="6" t="inlineStr">
@@ -2916,50 +2896,46 @@
       </x:c>
       <x:c r="B34" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-002</x:t>
+          <x:t>R-OCC-001</x:t>
         </x:is>
       </x:c>
       <x:c r="C34" s="3" t="inlineStr">
         <x:is>
-          <x:t>群体-个体下钻筛选</x:t>
+          <x:t>目标识别与维护</x:t>
         </x:is>
       </x:c>
       <x:c r="D34" s="6" t="str">
         <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
-      <x:c r="E34" s="3" t="inlineStr">
-        <x:is>
-          <x:t>结合人工智能算法实现从群体到个体的逐层下钻筛选，使情报分析人员能从大范围群体中按特征条件逐步缩小范围、定位到目标个体，支撑目标识别。</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F34" s="3" t="inlineStr">
-        <x:is>
-          <x:t>需求.md 社交媒体数据分析（群体下钻，V3.3 由 DC 移入）</x:t>
-        </x:is>
+      <x:c r="E34" s="3" t="str">
+        <x:v>识别舆情事件的目标要素并对其进行全生命周期维护。目标在系统中即数据对象——支持建档、修改、关联、状态流转与删除，而非一次识别即定型的只读结果。本能力融合情报侦察、多维画像与抓手挖掘中\"识别目标\"的部分：从舆情事件与传播数据中识别事件主体、传播源头、核心争议点、干预目标对象，并补充传播线索、事件/群体/账号/传播画像、干预切入点与薄弱点等目标属性，形成可持续维护的目标档案，为后续行动提供靶向。</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>需求.md 舆情行动（目标识别与维护）</x:v>
       </x:c>
       <x:c r="G34" s="3" t="inlineStr">
         <x:is>
-          <x:t>M-OCC-02 数据分析与情报（情报分析大脑）</x:t>
+          <x:t>M-OCC-01 目标档案与状态管理（目标数据管家）；M-OCC-03 目标关联网络（目标关系图谱）</x:t>
         </x:is>
       </x:c>
       <x:c r="H34" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-02-01</x:t>
+          <x:t>F-OCC-01-01；F-OCC-01-02；F-OCC-01-03；F-OCC-01-04；F-OCC-01-05；F-OCC-03-01；F-OCC-03-02</x:t>
         </x:is>
       </x:c>
       <x:c r="I34" s="3" t="inlineStr">
         <x:is>
-          <x:t>II-13 分析数据与情报接口（入，从 DC 取原始舆情/传播数据）。</x:t>
+          <x:t>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，经 R-OCC-002~005 分析后供目标识别融合）、EI-05 本地大模型推理（辅助识别）。</x:t>
         </x:is>
       </x:c>
       <x:c r="J34" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（筛选）</x:t>
+          <x:t>功能测试 + 演示（建档/修改/关联/状态流转）</x:t>
         </x:is>
       </x:c>
       <x:c r="K34" s="3" t="inlineStr">
         <x:is>
-          <x:t>给定群体特征条件，能经 AI 算法逐层下钻定位到目标个体；以人工标注的目标个体集合为基准，下钻结果的召回率不低于 70%、准确率不低于 80%（基准集规模与门槛在详细设计阶段确定）；算法异常时降级返回部分结果并告警。</x:t>
+          <x:t>目标可建档并赋予 target_id；目标各属性可新增、修改、删除；目标间可建立关联关系；目标状态可流转；目标档案可融合事件主体、传播、画像、切入点等多维信息；目标变更可经事件通知使用方；本期支持人工识别录入与系统数据维护。</x:t>
         </x:is>
       </x:c>
       <x:c r="L34" s="6" t="inlineStr">
@@ -2974,12 +2950,12 @@
       </x:c>
       <x:c r="B35" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-003</x:t>
+          <x:t>R-OCC-002</x:t>
         </x:is>
       </x:c>
       <x:c r="C35" s="3" t="inlineStr">
         <x:is>
-          <x:t>关系图谱与图查询</x:t>
+          <x:t>群体-个体下钻筛选</x:t>
         </x:is>
       </x:c>
       <x:c r="D35" s="6" t="str">
@@ -2987,12 +2963,12 @@
       </x:c>
       <x:c r="E35" s="3" t="inlineStr">
         <x:is>
-          <x:t>基于实体与关联数据绘制关系图谱并支持图查询，对给定实体输出关联拓扑与情报标签形成关联网络，使情报分析人员能看清目标实体的关系网络。</x:t>
+          <x:t>结合人工智能算法实现从群体到个体的逐层下钻筛选，使情报分析人员能从大范围群体中按特征条件逐步缩小范围、定位到目标个体，支撑目标识别。</x:t>
         </x:is>
       </x:c>
       <x:c r="F35" s="3" t="inlineStr">
         <x:is>
-          <x:t>需求.md 社交媒体数据分析（关系图谱，V3.3 由 DC 移入）</x:t>
+          <x:t>需求.md 社交媒体数据分析（群体下钻，V3.3 由 DC 移入）</x:t>
         </x:is>
       </x:c>
       <x:c r="G35" s="3" t="inlineStr">
@@ -3002,7 +2978,7 @@
       </x:c>
       <x:c r="H35" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-02-02</x:t>
+          <x:t>F-OCC-02-01</x:t>
         </x:is>
       </x:c>
       <x:c r="I35" s="3" t="inlineStr">
@@ -3012,12 +2988,12 @@
       </x:c>
       <x:c r="J35" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（图谱/图查询）</x:t>
+          <x:t>功能测试 + 演示（筛选）</x:t>
         </x:is>
       </x:c>
       <x:c r="K35" s="3" t="inlineStr">
         <x:is>
-          <x:t>给定实体能展示关系图谱并支持图查询；能输出关联拓扑与情报标签；查询数据量过大时分页或限流。</x:t>
+          <x:t>给定群体特征条件，能经 AI 算法逐层下钻定位到目标个体；以人工标注的目标个体集合为基准，下钻结果的召回率不低于 70%、准确率不低于 80%（基准集规模与门槛在详细设计阶段确定）；算法异常时降级返回部分结果并告警。</x:t>
         </x:is>
       </x:c>
       <x:c r="L35" s="6" t="inlineStr">
@@ -3032,12 +3008,12 @@
       </x:c>
       <x:c r="B36" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-004</x:t>
+          <x:t>R-OCC-003</x:t>
         </x:is>
       </x:c>
       <x:c r="C36" s="3" t="inlineStr">
         <x:is>
-          <x:t>实体检索与档案</x:t>
+          <x:t>关系图谱与图查询</x:t>
         </x:is>
       </x:c>
       <x:c r="D36" s="6" t="str">
@@ -3045,12 +3021,12 @@
       </x:c>
       <x:c r="E36" s="3" t="inlineStr">
         <x:is>
-          <x:t>提供基础信息检索（按账号、昵称、标识检索实体信息），并聚合多来源信息形成实体的全维度档案，使情报分析人员能快速定位实体并查看其完整画像。</x:t>
+          <x:t>基于实体与关联数据绘制关系图谱并支持图查询，对给定实体输出关联拓扑与情报标签形成关联网络，使情报分析人员能看清目标实体的关系网络。</x:t>
         </x:is>
       </x:c>
       <x:c r="F36" s="3" t="inlineStr">
         <x:is>
-          <x:t>需求.md 社交媒体数据分析（实体检索，V3.3 由 DC 移入）</x:t>
+          <x:t>需求.md 社交媒体数据分析（关系图谱，V3.3 由 DC 移入）</x:t>
         </x:is>
       </x:c>
       <x:c r="G36" s="3" t="inlineStr">
@@ -3060,7 +3036,7 @@
       </x:c>
       <x:c r="H36" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-02-03</x:t>
+          <x:t>F-OCC-02-02</x:t>
         </x:is>
       </x:c>
       <x:c r="I36" s="3" t="inlineStr">
@@ -3070,12 +3046,12 @@
       </x:c>
       <x:c r="J36" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（检索/档案）</x:t>
+          <x:t>功能测试 + 演示（图谱/图查询）</x:t>
         </x:is>
       </x:c>
       <x:c r="K36" s="3" t="inlineStr">
         <x:is>
-          <x:t>给定账号/昵称/标识能检索到实体信息；能聚合多来源信息形成全维度档案。</x:t>
+          <x:t>给定实体能展示关系图谱并支持图查询；能输出关联拓扑与情报标签；查询数据量过大时分页或限流。</x:t>
         </x:is>
       </x:c>
       <x:c r="L36" s="6" t="inlineStr">
@@ -3090,12 +3066,12 @@
       </x:c>
       <x:c r="B37" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-005</x:t>
+          <x:t>R-OCC-004</x:t>
         </x:is>
       </x:c>
       <x:c r="C37" s="3" t="inlineStr">
         <x:is>
-          <x:t>文本智能分析</x:t>
+          <x:t>实体检索与档案</x:t>
         </x:is>
       </x:c>
       <x:c r="D37" s="6" t="str">
@@ -3103,12 +3079,12 @@
       </x:c>
       <x:c r="E37" s="3" t="inlineStr">
         <x:is>
-          <x:t>对文本内容结合文本模型与关键词库进行规则匹配与分类筛选，用于内容研判与目标识别。文本模型调用底层 IRS 本地大模型，模型不可用时回退到关键词规则匹配。</x:t>
+          <x:t>提供基础信息检索（按账号、昵称、标识检索实体信息），并聚合多来源信息形成实体的全维度档案，使情报分析人员能快速定位实体并查看其完整画像。</x:t>
         </x:is>
       </x:c>
       <x:c r="F37" s="3" t="inlineStr">
         <x:is>
-          <x:t>需求.md 社交媒体数据分析（文本智能分析，V3.3 由 DC 移入）</x:t>
+          <x:t>需求.md 社交媒体数据分析（实体检索，V3.3 由 DC 移入）</x:t>
         </x:is>
       </x:c>
       <x:c r="G37" s="3" t="inlineStr">
@@ -3118,22 +3094,22 @@
       </x:c>
       <x:c r="H37" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-02-04</x:t>
+          <x:t>F-OCC-02-03</x:t>
         </x:is>
       </x:c>
       <x:c r="I37" s="3" t="inlineStr">
         <x:is>
-          <x:t>EI-05 本地大模型推理（调用 IRS 文本模型）、II-13 分析数据与情报接口（入，从 DC 取原始舆情/传播数据）、II-15 情报回注采集接口（出，向 DC 任务池 R-DC-007 提供分析产出）。</x:t>
+          <x:t>II-13 分析数据与情报接口（入，从 DC 取原始舆情/传播数据）。</x:t>
         </x:is>
       </x:c>
       <x:c r="J37" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（文本智能分析）</x:t>
+          <x:t>功能测试 + 演示（检索/档案）</x:t>
         </x:is>
       </x:c>
       <x:c r="K37" s="3" t="inlineStr">
         <x:is>
-          <x:t>给定文本能结合文本模型与关键词库输出分类筛选结果；以人工标注的测试文本集为基准，文本分类的宏平均 F1 不低于 0.75（基准集与门槛在详细设计阶段确定）；文本模型不可用时能回退到关键词规则匹配。</x:t>
+          <x:t>给定账号/昵称/标识能检索到实体信息；能聚合多来源信息形成全维度档案。</x:t>
         </x:is>
       </x:c>
       <x:c r="L37" s="6" t="inlineStr">
@@ -3148,40 +3124,50 @@
       </x:c>
       <x:c r="B38" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-006</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C38" s="3" t="str">
-        <x:v>行动编排</x:v>
+          <x:t>R-OCC-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="3" t="inlineStr">
+        <x:is>
+          <x:t>文本智能分析</x:t>
+        </x:is>
       </x:c>
       <x:c r="D38" s="6" t="str">
         <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
-      <x:c r="E38" s="3" t="str">
-        <x:v>根据目标档案与干预切入点匹配干预策略、生成作业方案，并以\"行动编排\"的方式直接编排群控子系统（MC）中的执行节点形成执行流程（图）落地，形成\"目标→编排→执行\"的闭环。OCC 直接编排 MC 中的节点，蜂群智能体子系统（SWM）作为\"智能体节点的供给方之一\"参与编排。编排的节点类型本期为两类——智能体节点（其智能体定义来源于 SWM 同步至 MC 的内容，见 R-MC-014）与自动化脚本节点。本期干预切入点与策略匹配以人工为主，系统提供方案生成与编排支撑。</x:v>
-      </x:c>
-      <x:c r="F38" s="3" t="str">
-        <x:v>需求.md 舆情行动（行动编排）</x:v>
-      </x:c>
-      <x:c r="G38" s="3" t="str">
-        <x:v>M-OCC-04 行动方案规划（行动参谋）；M-OCC-05 编排执行引擎（编排执行引擎）</x:v>
+      <x:c r="E38" s="3" t="inlineStr">
+        <x:is>
+          <x:t>对文本内容结合文本模型与关键词库进行规则匹配与分类筛选，用于内容研判与目标识别。文本模型调用底层 IRS 本地大模型，模型不可用时回退到关键词规则匹配。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="3" t="inlineStr">
+        <x:is>
+          <x:t>需求.md 社交媒体数据分析（文本智能分析，V3.3 由 DC 移入）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" s="3" t="inlineStr">
+        <x:is>
+          <x:t>M-OCC-02 数据分析与情报（情报分析大脑）</x:t>
+        </x:is>
       </x:c>
       <x:c r="H38" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-04-01；F-OCC-04-02；F-OCC-05-01；F-OCC-05-02；F-OCC-05-03</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I38" s="3" t="str">
-        <x:v>II-10 行动编排下发与执行回传接口。</x:v>
+          <x:t>F-OCC-02-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I38" s="3" t="inlineStr">
+        <x:is>
+          <x:t>EI-05 本地大模型推理（调用 IRS 文本模型）、II-13 分析数据与情报接口（入，从 DC 取原始舆情/传播数据）、II-15 情报回注采集接口（出，向 DC 任务池 R-DC-007 提供分析产出）。</x:t>
+        </x:is>
       </x:c>
       <x:c r="J38" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试 + 演示（节点编排落地经执行网关收口）</x:t>
+          <x:t>功能测试 + 演示（文本智能分析）</x:t>
         </x:is>
       </x:c>
       <x:c r="K38" s="3" t="inlineStr">
         <x:is>
-          <x:t>可根据目标档案匹配干预策略；可生成含内容、账号、时间、节奏的作业方案；可将 MC 中的智能体节点与自动化脚本节点编排为执行流程（图）；编排落地后动作经 MC 统一执行网关收口；节点类型后续可扩充。</x:t>
+          <x:t>给定文本能结合文本模型与关键词库输出分类筛选结果；以人工标注的测试文本集为基准，文本分类的宏平均 F1 不低于 0.75（基准集与门槛在详细设计阶段确定）；文本模型不可用时能回退到关键词规则匹配。</x:t>
         </x:is>
       </x:c>
       <x:c r="L38" s="6" t="inlineStr">
@@ -3196,41 +3182,41 @@
       </x:c>
       <x:c r="B39" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-007</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C39" s="3" t="inlineStr">
-        <x:is>
-          <x:t>效果评估</x:t>
-        </x:is>
+          <x:t>R-OCC-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>行动编排</x:v>
       </x:c>
       <x:c r="D39" s="6" t="str">
         <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E39" s="3" t="str">
-        <x:v>完成单轮干预成效统计、舆论走势修正、策略迭代反馈与作业复盘，并支持中短期与长期效果评估，形成行动闭环。本节的数据来源为两条：其一，数据爬取子系统（DC）的采集与分析结果（干预前后的舆情数据、传播数据、立场与情感变化）；其二，群控子系统（MC）可观测性能力（R-MC-010）上报的作业执行动作日志、任务日志与截图（投放触达、互动执行、账号行为记录）。OCC 基于这两类数据进行效果分析，不自行重复采集。</x:v>
+        <x:v>根据目标档案与干预切入点匹配干预策略、生成作业方案，并以\"行动编排\"的方式直接编排群控子系统（MC）中的执行节点形成执行流程（图）落地，形成\"目标→编排→执行\"的闭环。OCC 直接编排 MC 中的节点，蜂群智能体子系统（SWM）作为\"智能体节点的供给方之一\"参与编排。编排的节点类型本期为两类——智能体节点（其智能体定义来源于 SWM 同步至 MC 的内容，见 R-MC-014）与自动化脚本节点。本期干预切入点与策略匹配以人工为主，系统提供方案生成与编排支撑。</x:v>
       </x:c>
       <x:c r="F39" s="3" t="str">
-        <x:v>需求.md 舆情行动（效果评估）</x:v>
+        <x:v>需求.md 舆情行动（行动编排）</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
-        <x:v>M-OCC-06 效果评估（行动复盘官）</x:v>
+        <x:v>M-OCC-04 行动方案规划（行动参谋）；M-OCC-05 编排执行引擎（编排执行引擎）</x:v>
       </x:c>
       <x:c r="H39" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-06-01；F-OCC-06-02；F-OCC-06-03；F-OCC-06-04；F-OCC-06-05</x:t>
+          <x:t>F-OCC-04-01；F-OCC-04-02；F-OCC-05-01；F-OCC-05-02；F-OCC-05-03</x:t>
         </x:is>
       </x:c>
       <x:c r="I39" s="3" t="str">
-        <x:v>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，供 R-OCC-002~005 分析）、II-10 行动编排下发与执行回传（MC 作业数据来源）。</x:v>
+        <x:v>II-10 行动编排下发与执行回传接口。</x:v>
       </x:c>
       <x:c r="J39" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试（效果评估与策略迭代反馈）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K39" s="3" t="str">
-        <x:v>可基于 DC 舆情数据与 MC 作业数据进行单轮干预成效统计（成效定义为可计算指标：投放触达率、互动率、目标群体立场/情感正向偏移量，均以干预前后 DC 采集数据差值量化）；可修正评估舆论走势（走势修正偏差以人工复核一致率不低于 80% 为达标）；可将评估反馈策略库迭代；可结合 MC 作业记录作业复盘；可提供中短期与长期效果评估接口（各项指标的具体达标线在详细设计阶段按行动类型细化）。</x:v>
+          <x:t>功能测试 + 演示（节点编排落地经执行网关收口）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K39" s="3" t="inlineStr">
+        <x:is>
+          <x:t>可根据目标档案匹配干预策略；可生成含内容、账号、时间、节奏的作业方案；可将 MC 中的智能体节点与自动化脚本节点编排为执行流程（图）；编排落地后动作经 MC 统一执行网关收口；节点类型后续可扩充。</x:t>
+        </x:is>
       </x:c>
       <x:c r="L39" s="6" t="inlineStr">
         <x:is>
@@ -3244,47 +3230,41 @@
       </x:c>
       <x:c r="B40" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-008</x:t>
+          <x:t>R-OCC-007</x:t>
         </x:is>
       </x:c>
       <x:c r="C40" s="3" t="inlineStr">
         <x:is>
-          <x:t>舆论作业策略库</x:t>
+          <x:t>效果评估</x:t>
         </x:is>
       </x:c>
       <x:c r="D40" s="6" t="str">
         <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
       <x:c r="E40" s="3" t="str">
-        <x:v>搭建并迭代多语种、多场景、多风格的舆论作业策略库，为行动提供可复用、可演进的策略资产。</x:v>
+        <x:v>完成单轮干预成效统计、舆论走势修正、策略迭代反馈与作业复盘，并支持中短期与长期效果评估，形成行动闭环。本节的数据来源为两条：其一，数据爬取子系统（DC）的采集与分析结果（干预前后的舆情数据、传播数据、立场与情感变化）；其二，群控子系统（MC）可观测性能力（R-MC-010）上报的作业执行动作日志、任务日志与截图（投放触达、互动执行、账号行为记录）。OCC 基于这两类数据进行效果分析，不自行重复采集。</x:v>
       </x:c>
       <x:c r="F40" s="3" t="str">
-        <x:v>需求.md 舆情行动（策略库）</x:v>
-      </x:c>
-      <x:c r="G40" s="3" t="inlineStr">
-        <x:is>
-          <x:t>M-OCC-07 舆论作业策略库（策略资产库）</x:t>
-        </x:is>
+        <x:v>需求.md 舆情行动（效果评估）</x:v>
+      </x:c>
+      <x:c r="G40" s="3" t="str">
+        <x:v>M-OCC-06 效果评估（行动复盘官）</x:v>
       </x:c>
       <x:c r="H40" s="3" t="inlineStr">
         <x:is>
-          <x:t>F-OCC-07-01；F-OCC-07-02；F-OCC-07-03；F-OCC-07-04</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I40" s="3" t="inlineStr">
-        <x:is>
-          <x:t>无（策略库为 OCC 内部资产，供 R-OCC-006 编排调用）。</x:t>
-        </x:is>
+          <x:t>F-OCC-06-01；F-OCC-06-02；F-OCC-06-03；F-OCC-06-04；F-OCC-06-05</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I40" s="3" t="str">
+        <x:v>II-13 分析数据与情报接口（DC 原始舆情/传播数据→OCC，供 R-OCC-002~005 分析）、II-10 行动编排下发与执行回传（MC 作业数据来源）。</x:v>
       </x:c>
       <x:c r="J40" s="3" t="inlineStr">
         <x:is>
-          <x:t>功能测试（策略库）</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K40" s="3" t="inlineStr">
-        <x:is>
-          <x:t>策略库可按多语种多场景多风格组织；策略可分类管理与版本控制；可按效果反馈迭代优化（策略有效性以关联作业的效果评估结果 R-OCC-007 为判定依据，连续 3 轮作业成效未达标的策略标记为低效并进入淘汰候选）；可场景适配与动态调用。</x:t>
-        </x:is>
+          <x:t>功能测试（效果评估与策略迭代反馈）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K40" s="3" t="str">
+        <x:v>可基于 DC 舆情数据与 MC 作业数据进行单轮干预成效统计（成效定义为可计算指标：投放触达率、互动率、目标群体立场/情感正向偏移量，均以干预前后 DC 采集数据差值量化）；可修正评估舆论走势（走势修正偏差以人工复核一致率不低于 80% 为达标）；可将评估反馈策略库迭代；可结合 MC 作业记录作业复盘；可提供中短期与长期效果评估接口（各项指标的具体达标线在详细设计阶段按行动类型细化）。</x:v>
       </x:c>
       <x:c r="L40" s="6" t="inlineStr">
         <x:is>
@@ -3298,60 +3278,114 @@
       </x:c>
       <x:c r="B41" s="6" t="inlineStr">
         <x:is>
-          <x:t>R-OCC-009</x:t>
+          <x:t>R-OCC-008</x:t>
         </x:is>
       </x:c>
       <x:c r="C41" s="3" t="inlineStr">
         <x:is>
-          <x:t>内容资源管理</x:t>
+          <x:t>舆论作业策略库</x:t>
         </x:is>
       </x:c>
       <x:c r="D41" s="6" t="str">
         <x:v>OCC 舆情行动业务子系统</x:v>
       </x:c>
-      <x:c r="E41" s="3" t="inlineStr">
+      <x:c r="E41" s="3" t="str">
+        <x:v>搭建并迭代多语种、多场景、多风格的舆论作业策略库，为行动提供可复用、可演进的策略资产。</x:v>
+      </x:c>
+      <x:c r="F41" s="3" t="str">
+        <x:v>需求.md 舆情行动（策略库）</x:v>
+      </x:c>
+      <x:c r="G41" s="3" t="inlineStr">
+        <x:is>
+          <x:t>M-OCC-07 舆论作业策略库（策略资产库）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H41" s="3" t="inlineStr">
+        <x:is>
+          <x:t>F-OCC-07-01；F-OCC-07-02；F-OCC-07-03；F-OCC-07-04</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I41" s="3" t="inlineStr">
+        <x:is>
+          <x:t>无（策略库为 OCC 内部资产，供 R-OCC-006 编排调用）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J41" s="3" t="inlineStr">
+        <x:is>
+          <x:t>功能测试（策略库）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K41" s="3" t="inlineStr">
+        <x:is>
+          <x:t>策略库可按多语种多场景多风格组织；策略可分类管理与版本控制；可按效果反馈迭代优化（策略有效性以关联作业的效果评估结果 R-OCC-007 为判定依据，连续 3 轮作业成效未达标的策略标记为低效并进入淘汰候选）；可场景适配与动态调用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="L41" s="6" t="inlineStr">
+        <x:is>
+          <x:t>✓ 完整</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="6">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B42" s="6" t="inlineStr">
+        <x:is>
+          <x:t>R-OCC-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="3" t="inlineStr">
+        <x:is>
+          <x:t>内容资源管理</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="6" t="str">
+        <x:v>OCC 舆情行动业务子系统</x:v>
+      </x:c>
+      <x:c r="E42" s="3" t="inlineStr">
         <x:is>
           <x:t>承担内容资源的统一管理，作为内容主数据的唯一权威源，管理内容素材的入库、分类、审核与发布排期，并向各使用方主动分发内容标识（content_id）。蜂群智能体（SWM，养号文案）、群控（MC，内容投放）与未来 AI 素材制作为使用方，通过引用内容标识获取内容并维护各自的平台适配版本与使用记录。</x:t>
         </x:is>
       </x:c>
-      <x:c r="F41" s="3" t="inlineStr">
+      <x:c r="F42" s="3" t="inlineStr">
         <x:is>
           <x:t>开发方案 V1.1 内容模块（内容资源权威源）</x:t>
         </x:is>
       </x:c>
-      <x:c r="G41" s="3" t="inlineStr">
+      <x:c r="G42" s="3" t="inlineStr">
         <x:is>
           <x:t>M-OCC-08 内容主数据与排期（内容资源权威源）；M-OCC-09 内容审核与敏感词风控（内容合规守门人）</x:t>
         </x:is>
       </x:c>
-      <x:c r="H41" s="3" t="inlineStr">
+      <x:c r="H42" s="3" t="inlineStr">
         <x:is>
           <x:t>F-OCC-08-01；F-OCC-08-02；F-OCC-08-03；F-OCC-08-04；F-OCC-09-01；F-OCC-09-02</x:t>
         </x:is>
       </x:c>
-      <x:c r="I41" s="3" t="inlineStr">
+      <x:c r="I42" s="3" t="inlineStr">
         <x:is>
           <x:t>II-12 内容服务接口、II-12a 内容变更事件、EI-04 对象存储。</x:t>
         </x:is>
       </x:c>
-      <x:c r="J41" s="3" t="inlineStr">
+      <x:c r="J42" s="3" t="inlineStr">
         <x:is>
           <x:t>功能测试 + 演示（入库/分类/审核/排期/事件广播/分发）</x:t>
         </x:is>
       </x:c>
-      <x:c r="K41" s="3" t="inlineStr">
+      <x:c r="K42" s="3" t="inlineStr">
         <x:is>
           <x:t>内容主数据由本子系统唯一维护且使用方不复制；content_id 全局唯一可被各子系统引用；素材可分类管理与平台适配；发布排期可定时触发；内容可经审核与敏感词检测后发布；内容变更可经事件通知使用方并主动分发。</x:t>
         </x:is>
       </x:c>
-      <x:c r="L41" s="6" t="inlineStr">
+      <x:c r="L42" s="6" t="inlineStr">
         <x:is>
           <x:t>✓ 完整</x:t>
         </x:is>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:autoFilter ref="A1:L41"/>
+  <x:autoFilter ref="A1:L42"/>
   <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <x:pageSetup fitToWidth="1" fitToHeight="0" orientation="landscape"/>
 </x:worksheet>
@@ -5122,35 +5156,23 @@
           <x:t>内部接口 II</x:t>
         </x:is>
       </x:c>
-      <x:c r="C10" s="6" t="inlineStr">
-        <x:is>
-          <x:t>II-02</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>Agent 指令与日志接口</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>MC 服务端 ↔ 设备 Agent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>MC、Agent</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>入：下发指令；出：指令确认、日志与截图回传</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H10" s="3" t="inlineStr">
-        <x:is>
-          <x:t>R-MC-001/007</x:t>
-        </x:is>
+      <x:c r="C10" s="6" t="str">
+        <x:v>II-02（V4.1 / V3.10 改 Agent 长连接协议）</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>Agent 长连接协议（注册/心跳/占用/指令/媒体面协商）</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>MC M-MC-15.c 中心侧编排器 ↔ M-MC-15.a 设备主机侧 Agent</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>MC（M-MC-15）、Agent 主机进程</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>入：Agent 鉴权/心跳/动作结果/scrcpyReady；出：鉴权回应/runAction（ADB/无障碍）/occupy/release/startScrcpy</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>R-MC-015（V4.1 / V3.10 提供方调整，原 R-MC-001/007）</x:v>
       </x:c>
       <x:c r="I10" s="3" t="inlineStr">
         <x:is>

</xml_diff>